<commit_message>
Requirements template: Speak Up rename and the anonymity notice
Two requirements ERC raised, pre-filled as BR-002 and BR-003 on the
Other Requirements sheet. The notice text is ERC's, word for word.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/WB-Requirements-and-SLA-Template-v1.3.xlsx
+++ b/docs/WB-Requirements-and-SLA-Template-v1.3.xlsx
@@ -344,7 +344,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="285">
   <si>
     <t>Whistleblowing Reporting Portal - Requirements Template</t>
   </si>
@@ -705,6 +705,36 @@
     <t>Live in sandbox.</t>
   </si>
   <si>
+    <t>Intake / Portal</t>
+  </si>
+  <si>
+    <t>Rename the portal to "Speak Up"</t>
+  </si>
+  <si>
+    <t>Rename the portal from "Whistleblowing Reporting Portal" to "Speak Up" wherever reporters or staff see it: the help center portal name, the portal page title, the notification emails and the user guide.</t>
+  </si>
+  <si>
+    <t>The portal, the emails and the user guide show "Speak Up"; "Whistleblowing Reporting Portal" no longer appears anywhere a reporter or staff member can see it.</t>
+  </si>
+  <si>
+    <t>New</t>
+  </si>
+  <si>
+    <t>Portal name and emails are configuration only. The portal link does not change, so links already shared keep working.</t>
+  </si>
+  <si>
+    <t>Anonymity notice next to the anonymous option</t>
+  </si>
+  <si>
+    <t>Next to the anonymity selection option on the reporting form, show this statement: "Please note that choosing to remain anonymous may limit our ability to clarify facts or follow up with you during the investigation."</t>
+  </si>
+  <si>
+    <t>Opening the reporting form shows the statement, word for word, directly next to the anonymity option, before the reporter submits.</t>
+  </si>
+  <si>
+    <t>Shown as the help text of the anonymity option. Arabic text to confirm: "يرجى العلم بأن اختيار عدم الإفصاح عن هويتك قد يحدّ من قدرتنا على استيضاح الوقائع أو المتابعة معك أثناء التحقيق."</t>
+  </si>
+  <si>
     <t>Service Levels (SLA) and Escalation</t>
   </si>
   <si>
@@ -973,12 +1003,6 @@
   </si>
   <si>
     <t>GroupNames</t>
-  </si>
-  <si>
-    <t>Intake / Portal</t>
-  </si>
-  <si>
-    <t>New</t>
   </si>
   <si>
     <t>Working hours</t>
@@ -2054,7 +2078,7 @@
       </c>
       <c r="C29" s="8">
         <f>COUNTA('Other Requirements'!C7:C66)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="2:3" x14ac:dyDescent="0.3">
@@ -5261,39 +5285,63 @@
         <v>114</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="str">
         <f t="shared" ref="A7:A38" si="0">IF(C7="","","BR-"&amp;TEXT(ROW()-5,"000"))</f>
-        <v/>
-      </c>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
+        <v>BR-002</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>117</v>
+      </c>
       <c r="E7" s="14"/>
       <c r="F7" s="14"/>
       <c r="G7" s="14"/>
       <c r="H7" s="14"/>
-      <c r="I7" s="14"/>
+      <c r="I7" s="14" t="s">
+        <v>118</v>
+      </c>
       <c r="J7" s="17"/>
-      <c r="K7" s="14"/>
-      <c r="L7" s="14"/>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="K7" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="L7" s="14" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
+        <v>BR-003</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>122</v>
+      </c>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
       <c r="G8" s="14"/>
       <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
+      <c r="I8" s="14" t="s">
+        <v>123</v>
+      </c>
       <c r="J8" s="17"/>
-      <c r="K8" s="14"/>
-      <c r="L8" s="14"/>
+      <c r="K8" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="L8" s="14" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="str">
@@ -6342,7 +6390,7 @@
   <sheetData>
     <row r="1" spans="1:27" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="23" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="C1" s="24"/>
       <c r="D1" s="24"/>
@@ -6372,7 +6420,7 @@
     </row>
     <row r="2" spans="1:27" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="25" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="C2" s="24"/>
       <c r="D2" s="24"/>
@@ -6402,144 +6450,144 @@
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:27" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="M5" s="10" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="O5" s="10" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="Q5" s="10" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="R5" s="10" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="S5" s="10" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="T5" s="10" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="U5" s="10" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="V5" s="10" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="W5" s="10" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="X5" s="10" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="Y5" s="10" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="Z5" s="10" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="AA5" s="10" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6" spans="1:27" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="I6" s="11">
         <v>2</v>
       </c>
       <c r="J6" s="11" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="L6" s="18">
         <v>0.75</v>
       </c>
       <c r="M6" s="11" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="N6" s="11"/>
       <c r="O6" s="11">
         <v>0</v>
       </c>
       <c r="P6" s="11" t="s">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="Q6" s="11" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="R6" s="11" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="S6" s="11">
         <v>1</v>
@@ -6552,7 +6600,7 @@
       <c r="Y6" s="11"/>
       <c r="Z6" s="11"/>
       <c r="AA6" s="11" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
     </row>
     <row r="7" spans="1:27" ht="26.4" x14ac:dyDescent="0.3">
@@ -6561,34 +6609,34 @@
         <v>SLA-02</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="F7" s="19" t="s">
+        <v>172</v>
+      </c>
+      <c r="G7" s="19" t="s">
+        <v>173</v>
+      </c>
+      <c r="H7" s="19" t="s">
         <v>162</v>
-      </c>
-      <c r="G7" s="19" t="s">
-        <v>163</v>
-      </c>
-      <c r="H7" s="19" t="s">
-        <v>152</v>
       </c>
       <c r="I7" s="19">
         <v>2</v>
       </c>
       <c r="J7" s="19" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
       <c r="K7" s="19" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="L7" s="20"/>
       <c r="M7" s="19"/>
@@ -6597,13 +6645,13 @@
         <v>0</v>
       </c>
       <c r="P7" s="19" t="s">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="Q7" s="19" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="R7" s="19" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="S7" s="19"/>
       <c r="T7" s="19"/>
@@ -6614,7 +6662,7 @@
       <c r="Y7" s="19"/>
       <c r="Z7" s="19"/>
       <c r="AA7" s="19" t="s">
-        <v>164</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
@@ -8592,7 +8640,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="23" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="C1" s="24"/>
       <c r="D1" s="24"/>
@@ -8603,7 +8651,7 @@
     </row>
     <row r="2" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="25" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="C2" s="24"/>
       <c r="D2" s="24"/>
@@ -8614,67 +8662,67 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
       <c r="F6" s="11" t="s">
         <v>85</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A7" s="14" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
       <c r="C7" s="14"/>
       <c r="D7" s="14"/>
@@ -8685,10 +8733,10 @@
     </row>
     <row r="8" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="C8" s="14"/>
       <c r="D8" s="14"/>
@@ -8699,10 +8747,10 @@
     </row>
     <row r="9" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A9" s="14" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
       <c r="C9" s="14"/>
       <c r="D9" s="14"/>
@@ -8713,10 +8761,10 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
       <c r="C10" s="14"/>
       <c r="D10" s="14"/>
@@ -8727,10 +8775,10 @@
     </row>
     <row r="11" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
       <c r="C11" s="14"/>
       <c r="D11" s="14"/>
@@ -8741,10 +8789,10 @@
     </row>
     <row r="12" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A12" s="14" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="C12" s="14"/>
       <c r="D12" s="14"/>
@@ -8755,10 +8803,10 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="14" t="s">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="C13" s="14"/>
       <c r="D13" s="14"/>
@@ -8769,10 +8817,10 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="14" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
       <c r="C14" s="14"/>
       <c r="D14" s="14"/>
@@ -9338,72 +9386,72 @@
         <v>97</v>
       </c>
       <c r="C1" s="22" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="D1" s="22" t="s">
-        <v>196</v>
+        <v>206</v>
       </c>
       <c r="E1" s="22" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="F1" s="22" t="s">
-        <v>197</v>
+        <v>207</v>
       </c>
       <c r="G1" s="22" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="H1" s="22" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="I1" s="22" t="s">
-        <v>198</v>
+        <v>208</v>
       </c>
       <c r="J1" s="22" t="s">
-        <v>199</v>
+        <v>209</v>
       </c>
       <c r="K1" s="22" t="s">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="L1" s="22" t="s">
-        <v>201</v>
+        <v>211</v>
       </c>
       <c r="M1" s="22" t="s">
-        <v>202</v>
+        <v>212</v>
       </c>
       <c r="N1" s="22" t="s">
-        <v>203</v>
+        <v>213</v>
       </c>
       <c r="O1" s="22" t="s">
-        <v>204</v>
+        <v>214</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>205</v>
+        <v>115</v>
       </c>
       <c r="B2" t="s">
         <v>108</v>
       </c>
       <c r="C2" t="s">
-        <v>206</v>
+        <v>119</v>
       </c>
       <c r="D2" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="E2" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="F2" t="s">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="G2" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="H2" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="I2" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="J2" t="s">
         <v>85</v>
@@ -9415,136 +9463,136 @@
         <v>88</v>
       </c>
       <c r="M2" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="N2" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="O2" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="B3" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="C3" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="D3" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="E3" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="F3" t="s">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="G3" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
       <c r="H3" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="I3" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="J3" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="K3" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="L3" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="M3" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="N3" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="O3" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="B4" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="C4" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="D4" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="E4" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="F4" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="G4" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="I4" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="K4" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="M4" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="N4" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="O4" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="B5" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="C5" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="D5" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="E5" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="F5" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="G5" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="I5" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="K5" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="M5" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="N5" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="O5" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
@@ -9555,150 +9603,150 @@
         <v>113</v>
       </c>
       <c r="D6" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="E6" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="F6" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="K6" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="M6" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="N6" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="O6" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="D7" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="F7" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="M7" t="s">
         <v>84</v>
       </c>
       <c r="N7" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="O7" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="D8" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="M8" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="N8" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="O8" t="s">
-        <v>156</v>
+        <v>166</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="D9" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="M9" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="N9" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="O9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="D10" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="M10" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="N10" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="D11" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="M11" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="N11" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="D12" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="M12" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="N12" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M13" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
       <c r="N13" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M14" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="N14" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M15" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
       <c r="N15" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M16" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
       <c r="N16" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Requirements template: "What can I report?" guidance
BR-004 asks for the reportable-matters guidance behind an info button
rather than as text on the form; BR-005 holds ERC's guidance text word
for word. The notes say plainly that Jira's portal has no native popup.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/WB-Requirements-and-SLA-Template-v1.3.xlsx
+++ b/docs/WB-Requirements-and-SLA-Template-v1.3.xlsx
@@ -344,7 +344,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="293">
   <si>
     <t>Whistleblowing Reporting Portal - Requirements Template</t>
   </si>
@@ -733,6 +733,42 @@
   </si>
   <si>
     <t>Shown as the help text of the anonymity option. Arabic text to confirm: "يرجى العلم بأن اختيار عدم الإفصاح عن هويتك قد يحدّ من قدرتنا على استيضاح الوقائع أو المتابعة معك أثناء التحقيق."</t>
+  </si>
+  <si>
+    <t>"What can I report?" guidance behind an info button</t>
+  </si>
+  <si>
+    <t>The portal should present a summary of reportable matters to guide reporters. It must not be static text on the form: an info icon or button (e.g. "What can I report?" or an "i" next to the title) opens the guidance in BR-005 as an expandable panel, popup or tooltip, and it can be collapsed again so it does not clutter the form.</t>
+  </si>
+  <si>
+    <t>The form shows only the button; clicking or tapping it shows the BR-005 text in full; it can be closed again; it works on desktop and mobile.</t>
+  </si>
+  <si>
+    <t>Jira's portal has no native info-icon popup. Closest standard option: a "What can I report?" toggle on the form that shows and hides a section holding the text. A true icon or popup needs a portal customization - to agree with ERC.</t>
+  </si>
+  <si>
+    <t>Reportable matters - guidance text</t>
+  </si>
+  <si>
+    <t>Text to show in the "What can I report?" guidance (BR-004), word for word:
+A report may concern wrongdoing that has occurred, is occurring, or is likely to occur. Reportable matters include, without limitation:
+Fraud, theft, embezzlement, misappropriation or misuse of assets, funds or information.
+Bribery, kickbacks, facilitation payments, trading in influence, extortion or any other form of corruption.
+Money laundering, terrorist financing, sanctions evasion or suspicious financial activity.
+Collusion, bid rigging, conflict of interest, favoritism or abuse of position in procurement, contracting, land, permitting, licensing or recruitment decisions.
+Falsification, concealment, destruction or manipulation of records, accounts, reports or evidence.
+Breach of law, regulation, license conditions, contractual obligation or internal policy.
+Harassment, bullying, discrimination, abuse of authority or other serious workplace misconduct.
+Health, safety or environmental danger, and breaches of construction, heritage or site-protection requirements.
+Information security breaches, unauthorized disclosure of confidential or personal data, and misuse of systems.
+Deliberate circumvention or override of internal controls.
+Retaliation against a whistleblower, witness or any person assisting a case, or any attempt to obstruct or interfere with a case.</t>
+  </si>
+  <si>
+    <t>The guidance shows this text word for word, including all eleven items.</t>
+  </si>
+  <si>
+    <t>Arabic version to be provided or confirmed by ERC, as the form is bilingual.</t>
   </si>
   <si>
     <t>Service Levels (SLA) and Escalation</t>
@@ -2078,7 +2114,7 @@
       </c>
       <c r="C29" s="8">
         <f>COUNTA('Other Requirements'!C7:C66)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30" spans="2:3" x14ac:dyDescent="0.3">
@@ -5343,39 +5379,63 @@
         <v>124</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" ht="92.4" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
+        <v>BR-004</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>126</v>
+      </c>
       <c r="E9" s="14"/>
       <c r="F9" s="14"/>
       <c r="G9" s="14"/>
       <c r="H9" s="14"/>
-      <c r="I9" s="14"/>
+      <c r="I9" s="14" t="s">
+        <v>127</v>
+      </c>
       <c r="J9" s="17"/>
-      <c r="K9" s="14"/>
-      <c r="L9" s="14"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="K9" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="L9" s="14" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
+        <v>BR-005</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>130</v>
+      </c>
       <c r="E10" s="14"/>
       <c r="F10" s="14"/>
       <c r="G10" s="14"/>
       <c r="H10" s="14"/>
-      <c r="I10" s="14"/>
+      <c r="I10" s="14" t="s">
+        <v>131</v>
+      </c>
       <c r="J10" s="17"/>
-      <c r="K10" s="14"/>
-      <c r="L10" s="14"/>
+      <c r="K10" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="L10" s="14" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="13" t="str">
@@ -6390,7 +6450,7 @@
   <sheetData>
     <row r="1" spans="1:27" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="23" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="C1" s="24"/>
       <c r="D1" s="24"/>
@@ -6420,7 +6480,7 @@
     </row>
     <row r="2" spans="1:27" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="25" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="C2" s="24"/>
       <c r="D2" s="24"/>
@@ -6450,144 +6510,144 @@
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:27" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="M5" s="10" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="O5" s="10" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="Q5" s="10" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="R5" s="10" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="S5" s="10" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="T5" s="10" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="U5" s="10" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="V5" s="10" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="W5" s="10" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="X5" s="10" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="Y5" s="10" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="Z5" s="10" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="AA5" s="10" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:27" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="I6" s="11">
         <v>2</v>
       </c>
       <c r="J6" s="11" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="L6" s="18">
         <v>0.75</v>
       </c>
       <c r="M6" s="11" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="N6" s="11"/>
       <c r="O6" s="11">
         <v>0</v>
       </c>
       <c r="P6" s="11" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="Q6" s="11" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="R6" s="11" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="S6" s="11">
         <v>1</v>
@@ -6600,7 +6660,7 @@
       <c r="Y6" s="11"/>
       <c r="Z6" s="11"/>
       <c r="AA6" s="11" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
     </row>
     <row r="7" spans="1:27" ht="26.4" x14ac:dyDescent="0.3">
@@ -6609,34 +6669,34 @@
         <v>SLA-02</v>
       </c>
       <c r="B7" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>179</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>166</v>
+      </c>
+      <c r="E7" s="19" t="s">
+        <v>167</v>
+      </c>
+      <c r="F7" s="19" t="s">
+        <v>180</v>
+      </c>
+      <c r="G7" s="19" t="s">
+        <v>181</v>
+      </c>
+      <c r="H7" s="19" t="s">
         <v>170</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>171</v>
-      </c>
-      <c r="D7" s="19" t="s">
-        <v>158</v>
-      </c>
-      <c r="E7" s="19" t="s">
-        <v>159</v>
-      </c>
-      <c r="F7" s="19" t="s">
-        <v>172</v>
-      </c>
-      <c r="G7" s="19" t="s">
-        <v>173</v>
-      </c>
-      <c r="H7" s="19" t="s">
-        <v>162</v>
       </c>
       <c r="I7" s="19">
         <v>2</v>
       </c>
       <c r="J7" s="19" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="K7" s="19" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="L7" s="20"/>
       <c r="M7" s="19"/>
@@ -6645,13 +6705,13 @@
         <v>0</v>
       </c>
       <c r="P7" s="19" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="Q7" s="19" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="R7" s="19" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="S7" s="19"/>
       <c r="T7" s="19"/>
@@ -6662,7 +6722,7 @@
       <c r="Y7" s="19"/>
       <c r="Z7" s="19"/>
       <c r="AA7" s="19" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
@@ -8640,7 +8700,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="23" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="C1" s="24"/>
       <c r="D1" s="24"/>
@@ -8651,7 +8711,7 @@
     </row>
     <row r="2" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="25" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="C2" s="24"/>
       <c r="D2" s="24"/>
@@ -8662,67 +8722,67 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="F6" s="11" t="s">
         <v>85</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A7" s="14" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="C7" s="14"/>
       <c r="D7" s="14"/>
@@ -8733,10 +8793,10 @@
     </row>
     <row r="8" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="C8" s="14"/>
       <c r="D8" s="14"/>
@@ -8747,10 +8807,10 @@
     </row>
     <row r="9" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A9" s="14" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="C9" s="14"/>
       <c r="D9" s="14"/>
@@ -8761,10 +8821,10 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="C10" s="14"/>
       <c r="D10" s="14"/>
@@ -8775,10 +8835,10 @@
     </row>
     <row r="11" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="C11" s="14"/>
       <c r="D11" s="14"/>
@@ -8789,10 +8849,10 @@
     </row>
     <row r="12" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A12" s="14" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="C12" s="14"/>
       <c r="D12" s="14"/>
@@ -8803,10 +8863,10 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="14" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="C13" s="14"/>
       <c r="D13" s="14"/>
@@ -8817,10 +8877,10 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="14" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="C14" s="14"/>
       <c r="D14" s="14"/>
@@ -9386,43 +9446,43 @@
         <v>97</v>
       </c>
       <c r="C1" s="22" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="D1" s="22" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="E1" s="22" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="F1" s="22" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="G1" s="22" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="H1" s="22" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I1" s="22" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="J1" s="22" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="K1" s="22" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="L1" s="22" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="M1" s="22" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="N1" s="22" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="O1" s="22" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
@@ -9436,22 +9496,22 @@
         <v>119</v>
       </c>
       <c r="D2" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="E2" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="F2" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="G2" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="H2" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="I2" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="J2" t="s">
         <v>85</v>
@@ -9463,136 +9523,136 @@
         <v>88</v>
       </c>
       <c r="M2" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="N2" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="O2" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="B3" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="C3" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="D3" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="E3" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="F3" t="s">
+        <v>179</v>
+      </c>
+      <c r="G3" t="s">
         <v>171</v>
       </c>
-      <c r="G3" t="s">
-        <v>163</v>
-      </c>
       <c r="H3" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="I3" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="J3" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="K3" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="L3" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="M3" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="N3" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="O3" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="B4" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="C4" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="D4" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="E4" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="F4" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="G4" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="I4" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="K4" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="M4" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="N4" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="O4" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="B5" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="C5" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="D5" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="E5" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="F5" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="G5" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="I5" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="K5" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="M5" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="N5" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="O5" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
@@ -9603,150 +9663,150 @@
         <v>113</v>
       </c>
       <c r="D6" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="E6" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="F6" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="K6" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="M6" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="N6" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="O6" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="D7" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="F7" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="M7" t="s">
         <v>84</v>
       </c>
       <c r="N7" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="O7" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="D8" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="M8" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="N8" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="O8" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="D9" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="M9" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="N9" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="O9" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="D10" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
       <c r="M10" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="N10" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="D11" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="M11" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
       <c r="N11" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="D12" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="M12" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
       <c r="N12" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M13" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="N13" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M14" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="N14" t="s">
-        <v>280</v>
+        <v>288</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M15" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="N15" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M16" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="N16" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Requirements template: escalation branch to Internal Audit (BR-006)
Two questions on the reporting page send reports about the Board, GRC
or Cybersecurity straight to Internal Audit. A new 'BR-006 Impact' sheet
lists the eleven areas of today's setup this touches and the decisions
ERC needs to make, with a cell for each answer.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/WB-Requirements-and-SLA-Template-v1.3.xlsx
+++ b/docs/WB-Requirements-and-SLA-Template-v1.3.xlsx
@@ -11,9 +11,10 @@
     <sheet name="Service Catalog" sheetId="2" r:id="rId2"/>
     <sheet name="Request Form Fields" sheetId="3" r:id="rId3"/>
     <sheet name="Other Requirements" sheetId="4" r:id="rId4"/>
-    <sheet name="SLA" sheetId="5" r:id="rId5"/>
-    <sheet name="Groups &amp; Contacts" sheetId="6" r:id="rId6"/>
-    <sheet name="Lists" sheetId="7" state="hidden" r:id="rId7"/>
+    <sheet name="BR-006 Impact" sheetId="5" r:id="rId5"/>
+    <sheet name="SLA" sheetId="6" r:id="rId6"/>
+    <sheet name="Groups &amp; Contacts" sheetId="7" r:id="rId7"/>
+    <sheet name="Lists" sheetId="8" state="hidden" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="Area">Lists!$A$2:$A$11</definedName>
@@ -344,7 +345,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="343">
   <si>
     <t>Whistleblowing Reporting Portal - Requirements Template</t>
   </si>
@@ -398,6 +399,12 @@
   </si>
   <si>
     <t>Anything that is not a service or a field: notifications, reports, access rules, data retention.</t>
+  </si>
+  <si>
+    <t>BR-006 Impact</t>
+  </si>
+  <si>
+    <t>What the escalation branch (BR-006) changes in today's setup, and the decisions needed - answer in the yellow 'ERC answer' cells.</t>
   </si>
   <si>
     <t>SLA</t>
@@ -771,6 +778,163 @@
     <t>Arabic version to be provided or confirmed by ERC, as the form is bilingual.</t>
   </si>
   <si>
+    <t>Routing</t>
+  </si>
+  <si>
+    <t>Escalation questions on the reporting page (new Internal Audit branch)</t>
+  </si>
+  <si>
+    <t>Add two questions to the reporting page. This changes the existing workflow and adds a new branch.
+Q1: "Is the reported case related to the Board of Directors?"
+- Yes: the report goes to the Internal Audit team. Flow: Reject, or Under Investigation and then Closed.
+- No: ask Q2.
+Q2: "Is it related to the Governance, Risk &amp; Compliance or Cybersecurity department?"
+- Yes: the report goes to Internal Audit.
+- No: continue with the normal workflow.
+Impact on current areas: see the 'BR-006 Impact' sheet.</t>
+  </si>
+  <si>
+    <t>A Yes to either question sends the report straight to Internal Audit, with no Compliance review, and GRC-Compliance can neither see it nor receive an email about it. A No to both follows today's workflow unchanged.</t>
+  </si>
+  <si>
+    <t>11 impacted areas and the decisions ERC needs to make are listed on the 'BR-006 Impact' sheet.</t>
+  </si>
+  <si>
+    <t>BR-006 - Impact of the escalation branch</t>
+  </si>
+  <si>
+    <t>What changes in the current setup when a report concerns the Board, GRC or Cybersecurity</t>
+  </si>
+  <si>
+    <t>Escalated reports concern GRC itself, so the rule behind most rows is: nothing about them may reach GRC-Compliance - not the report, not an email, not an SLA escalation.</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>Today</t>
+  </si>
+  <si>
+    <t>Change needed</t>
+  </si>
+  <si>
+    <t>Decision needed from ERC</t>
+  </si>
+  <si>
+    <t>ERC answer</t>
+  </si>
+  <si>
+    <t>Reporting form</t>
+  </si>
+  <si>
+    <t>One request type: summary, phone number, details, attachments and the pre-filled anonymous email.</t>
+  </si>
+  <si>
+    <t>Add the two Yes/No questions (English and Arabic). Q2 shows only when Q1 is No. Both mandatory. The conditional question needs a form on the portal.</t>
+  </si>
+  <si>
+    <t>Confirm the Arabic wording and that both questions are mandatory.</t>
+  </si>
+  <si>
+    <t>Workflow</t>
+  </si>
+  <si>
+    <t>Open -&gt; Compliance review -&gt; Under Investigation -&gt; Investigation Approved. A team rejection goes Back to Compliance.</t>
+  </si>
+  <si>
+    <t>New branch for escalated reports: Open -&gt; Under Investigation (Internal Audit) -&gt; Closed, or Rejected with a reason. No path back to Compliance on this branch.</t>
+  </si>
+  <si>
+    <t>Should Internal Audit record an Investigation Outcome when closing, as on the normal branch?</t>
+  </si>
+  <si>
+    <t>Routing (automation)</t>
+  </si>
+  <si>
+    <t>The investigation group is set from the Report Category when the Compliance Manager approves.</t>
+  </si>
+  <si>
+    <t>New rule on submission: if either answer is Yes, assign Internal Audit at once and skip Compliance review. Today's routing rule is unchanged for the normal branch.</t>
+  </si>
+  <si>
+    <t>Confidentiality (issue security)</t>
+  </si>
+  <si>
+    <t>GRC-Compliance can see every report. FollowUP TKT sees all reports.</t>
+  </si>
+  <si>
+    <t>Escalated reports get a new security level that GRC-Compliance cannot see (Internal Audit only).</t>
+  </si>
+  <si>
+    <t>Who else may see escalated reports (e.g. the Audit Committee)? Should FollowUP TKT still see them?</t>
+  </si>
+  <si>
+    <t>Every new report emails GRC-Compliance. The reporter gets an acknowledgement.</t>
+  </si>
+  <si>
+    <t>Escalated reports email Internal Audit only; the GRC new-report rule must skip them. The reporter's acknowledgement does not change.</t>
+  </si>
+  <si>
+    <t>SLA and escalation</t>
+  </si>
+  <si>
+    <t>Compliance decision: 2 working days. Investigation decision: 2 working days. Breaches email HO-Compliance.</t>
+  </si>
+  <si>
+    <t>The Compliance SLA does not apply. Breaches on escalated reports must not go to HO-Compliance.</t>
+  </si>
+  <si>
+    <t>Who receives SLA escalations for escalated reports? Is 2 working days right for Internal Audit's decision?</t>
+  </si>
+  <si>
+    <t>Classification</t>
+  </si>
+  <si>
+    <t>The Compliance Manager records the Report Category in the Compliance Approval form.</t>
+  </si>
+  <si>
+    <t>Escalated reports skip that form, so no Report Category is recorded unless Internal Audit sets it.</t>
+  </si>
+  <si>
+    <t>Should Internal Audit classify escalated reports, so they appear in the statistics by category?</t>
+  </si>
+  <si>
+    <t>Queues and reporting (incl. Power BI)</t>
+  </si>
+  <si>
+    <t>Queues and reports cover all reports, by category.</t>
+  </si>
+  <si>
+    <t>New queue: Escalated - Internal Audit. Reports and Power BI see escalated cases only if their account is allowed on the new security level.</t>
+  </si>
+  <si>
+    <t>Should escalated cases appear in management reporting, and in how much detail?</t>
+  </si>
+  <si>
+    <t>Reports about Internal Audit</t>
+  </si>
+  <si>
+    <t>The two questions do not cover a report about Internal Audit itself; it would follow the normal flow to GRC.</t>
+  </si>
+  <si>
+    <t>Is that acceptable, or is a third question needed?</t>
+  </si>
+  <si>
+    <t>Documentation and training</t>
+  </si>
+  <si>
+    <t>User guide v1.1, workflow diagram and SLA template describe one branch.</t>
+  </si>
+  <si>
+    <t>Update the guide, the diagram and the SLA template; brief Internal Audit on the new branch.</t>
+  </si>
+  <si>
+    <t>Reports already submitted</t>
+  </si>
+  <si>
+    <t>No change: the questions apply to new reports only.</t>
+  </si>
+  <si>
     <t>Service Levels (SLA) and Escalation</t>
   </si>
   <si>
@@ -1050,9 +1214,6 @@
     <t>Short text (Text Field - single line)</t>
   </si>
   <si>
-    <t>Classification</t>
-  </si>
-  <si>
     <t>Should have</t>
   </si>
   <si>
@@ -1081,9 +1242,6 @@
   </si>
   <si>
     <t>Paragraph (Text Field - multi-line)</t>
-  </si>
-  <si>
-    <t>Routing</t>
   </si>
   <si>
     <t>Could have</t>
@@ -1255,7 +1413,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1317,6 +1475,12 @@
       <color rgb="FF5E716B"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1D2B27"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -1373,7 +1537,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1412,6 +1576,24 @@
     <xf numFmtId="14" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="9" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1429,11 +1611,11 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1609,6 +1791,38 @@
 </file>
 
 <file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="438150" cy="390525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
@@ -1928,7 +2142,7 @@
   <sheetPr>
     <tabColor rgb="FF024638"/>
   </sheetPr>
-  <dimension ref="B1:C34"/>
+  <dimension ref="B1:C35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1937,16 +2151,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:3" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="24"/>
+      <c r="C1" s="30"/>
     </row>
     <row r="2" spans="2:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="24"/>
+      <c r="C2" s="30"/>
     </row>
     <row r="4" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
@@ -2022,7 +2236,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:3" ht="26.4" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>20</v>
       </c>
@@ -2030,16 +2244,16 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B17" s="1" t="s">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B16" s="5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B18" s="5" t="s">
+      <c r="C16" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="6" t="s">
+    </row>
+    <row r="18" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B18" s="1" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2071,90 +2285,98 @@
       <c r="B22" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C22" s="7"/>
+      <c r="C22" s="6" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B23" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C23" s="7"/>
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B24" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C24" s="7"/>
     </row>
-    <row r="26" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B26" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B27" s="5" t="s">
+    <row r="25" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B25" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C25" s="7"/>
+    </row>
+    <row r="27" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B27" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B28" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C28" s="8">
         <f>COUNTA('Service Catalog'!C7:C66)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B28" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C28" s="8">
+    <row r="29" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B29" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C29" s="8">
         <f>COUNTA('Request Form Fields'!D7:D66)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B29" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="C29" s="8">
-        <f>COUNTA('Other Requirements'!C7:C66)</f>
-        <v>4</v>
-      </c>
-    </row>
     <row r="30" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B30" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C30" s="8">
+        <f>COUNTA('Other Requirements'!C7:C66)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B31" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C31" s="8">
         <f>COUNTIF('Other Requirements'!K7:K66,"Approved")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B31" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C31" s="8">
+    <row r="32" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B32" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C32" s="8">
         <f>COUNTA(SLA!B7:B66)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B32" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="C32" s="8">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B33" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C33" s="8">
         <f>COUNTA('Groups &amp; Contacts'!C7:C66)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B34" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="C34" s="27"/>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B35" s="31" t="s">
+        <v>43</v>
+      </c>
+      <c r="C35" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B35:C35"/>
     <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B34:C34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -2183,121 +2405,121 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-      <c r="M1" s="24"/>
-      <c r="N1" s="24"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="30"/>
+      <c r="N1" s="30"/>
     </row>
     <row r="2" spans="1:14" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="25" t="s">
-        <v>42</v>
-      </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
-      <c r="L2" s="24"/>
-      <c r="M2" s="24"/>
-      <c r="N2" s="24"/>
+      <c r="B2" s="33" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
+      <c r="M2" s="30"/>
+      <c r="N2" s="30"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M5" s="10" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="J6" s="11" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L6" s="12">
         <f t="shared" ref="L6:L37" si="0">IF(C6="","",SUMPRODUCT((TRIM(F6:H6)&lt;&gt;"")*(TRIM(F6:H6)&lt;&gt;"None")*(TRIM(F6:H6)&lt;&gt;"-")))</f>
@@ -2308,7 +2530,7 @@
         <v>1</v>
       </c>
       <c r="N6" s="11" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
@@ -3850,115 +4072,115 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
     </row>
     <row r="2" spans="1:12" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="25" t="s">
-        <v>69</v>
-      </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
-      <c r="L2" s="24"/>
+      <c r="B2" s="33" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C6" s="11">
         <v>1</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="J6" s="11" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="K6" s="11" t="str">
         <f t="shared" ref="K6:K37" si="0">IF(F6="","",IFERROR(INDEX(JiraField,MATCH(F6,FieldType,0)),"Ejada to review"))</f>
         <v>Select List (single choice)</v>
       </c>
       <c r="L6" s="11" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
@@ -5211,114 +5433,114 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
     </row>
     <row r="2" spans="1:12" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
-      <c r="L2" s="24"/>
+      <c r="B2" s="33" t="s">
+        <v>92</v>
+      </c>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="J6" s="16" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="L6" s="11" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="52.8" x14ac:dyDescent="0.3">
@@ -5327,27 +5549,27 @@
         <v>BR-002</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E7" s="14"/>
       <c r="F7" s="14"/>
       <c r="G7" s="14"/>
       <c r="H7" s="14"/>
       <c r="I7" s="14" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="J7" s="17"/>
       <c r="K7" s="14" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="L7" s="14" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="79.2" x14ac:dyDescent="0.3">
@@ -5356,27 +5578,27 @@
         <v>BR-003</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
       <c r="G8" s="14"/>
       <c r="H8" s="14"/>
       <c r="I8" s="14" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="J8" s="17"/>
       <c r="K8" s="14" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="L8" s="14" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="92.4" x14ac:dyDescent="0.3">
@@ -5385,27 +5607,27 @@
         <v>BR-004</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E9" s="14"/>
       <c r="F9" s="14"/>
       <c r="G9" s="14"/>
       <c r="H9" s="14"/>
       <c r="I9" s="14" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J9" s="17"/>
       <c r="K9" s="14" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="L9" s="14" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="409.6" x14ac:dyDescent="0.3">
@@ -5414,45 +5636,57 @@
         <v>BR-005</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E10" s="14"/>
       <c r="F10" s="14"/>
       <c r="G10" s="14"/>
       <c r="H10" s="14"/>
       <c r="I10" s="14" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="J10" s="17"/>
       <c r="K10" s="14" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="L10" s="14" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="184.8" x14ac:dyDescent="0.3">
       <c r="A11" s="13" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
+        <v>BR-006</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>137</v>
+      </c>
       <c r="E11" s="14"/>
       <c r="F11" s="14"/>
       <c r="G11" s="14"/>
       <c r="H11" s="14"/>
-      <c r="I11" s="14"/>
+      <c r="I11" s="14" t="s">
+        <v>138</v>
+      </c>
       <c r="J11" s="17"/>
-      <c r="K11" s="14"/>
-      <c r="L11" s="14"/>
+      <c r="K11" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="L11" s="14" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="str">
@@ -6415,6 +6649,273 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FF024638"/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="42" customWidth="1"/>
+    <col min="4" max="4" width="52" customWidth="1"/>
+    <col min="5" max="5" width="46" customWidth="1"/>
+    <col min="6" max="6" width="40" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+    </row>
+    <row r="2" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="33" t="s">
+        <v>141</v>
+      </c>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="E5" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="F5" s="18" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="19">
+        <v>1</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>149</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>150</v>
+      </c>
+      <c r="E6" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="F6" s="14"/>
+    </row>
+    <row r="7" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="21">
+        <v>2</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>153</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>154</v>
+      </c>
+      <c r="E7" s="21" t="s">
+        <v>155</v>
+      </c>
+      <c r="F7" s="14"/>
+    </row>
+    <row r="8" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="19">
+        <v>3</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>156</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="E8" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="F8" s="23"/>
+    </row>
+    <row r="9" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="21">
+        <v>4</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>159</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>160</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>161</v>
+      </c>
+      <c r="E9" s="21" t="s">
+        <v>162</v>
+      </c>
+      <c r="F9" s="14"/>
+    </row>
+    <row r="10" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="19">
+        <v>5</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>163</v>
+      </c>
+      <c r="D10" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="E10" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="F10" s="23"/>
+    </row>
+    <row r="11" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="21">
+        <v>6</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>166</v>
+      </c>
+      <c r="D11" s="21" t="s">
+        <v>167</v>
+      </c>
+      <c r="E11" s="21" t="s">
+        <v>168</v>
+      </c>
+      <c r="F11" s="14"/>
+    </row>
+    <row r="12" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A12" s="19">
+        <v>7</v>
+      </c>
+      <c r="B12" s="20" t="s">
+        <v>169</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>170</v>
+      </c>
+      <c r="D12" s="19" t="s">
+        <v>171</v>
+      </c>
+      <c r="E12" s="19" t="s">
+        <v>172</v>
+      </c>
+      <c r="F12" s="14"/>
+    </row>
+    <row r="13" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="21">
+        <v>8</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>173</v>
+      </c>
+      <c r="C13" s="21" t="s">
+        <v>174</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>175</v>
+      </c>
+      <c r="E13" s="21" t="s">
+        <v>176</v>
+      </c>
+      <c r="F13" s="14"/>
+    </row>
+    <row r="14" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A14" s="19">
+        <v>9</v>
+      </c>
+      <c r="B14" s="20" t="s">
+        <v>177</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="D14" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="E14" s="19" t="s">
+        <v>179</v>
+      </c>
+      <c r="F14" s="14"/>
+    </row>
+    <row r="15" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A15" s="21">
+        <v>10</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>180</v>
+      </c>
+      <c r="C15" s="21" t="s">
+        <v>181</v>
+      </c>
+      <c r="D15" s="21" t="s">
+        <v>182</v>
+      </c>
+      <c r="E15" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="F15" s="23"/>
+    </row>
+    <row r="16" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A16" s="19">
+        <v>11</v>
+      </c>
+      <c r="B16" s="20" t="s">
+        <v>183</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="D16" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="E16" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="F16" s="23"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF024638"/>
@@ -6449,205 +6950,205 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="23" t="s">
-        <v>133</v>
-      </c>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-      <c r="M1" s="24"/>
-      <c r="N1" s="24"/>
-      <c r="O1" s="24"/>
-      <c r="P1" s="24"/>
-      <c r="Q1" s="24"/>
-      <c r="R1" s="24"/>
-      <c r="S1" s="24"/>
-      <c r="T1" s="24"/>
-      <c r="U1" s="24"/>
-      <c r="V1" s="24"/>
-      <c r="W1" s="24"/>
-      <c r="X1" s="24"/>
-      <c r="Y1" s="24"/>
-      <c r="Z1" s="24"/>
-      <c r="AA1" s="24"/>
+      <c r="B1" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="30"/>
+      <c r="N1" s="30"/>
+      <c r="O1" s="30"/>
+      <c r="P1" s="30"/>
+      <c r="Q1" s="30"/>
+      <c r="R1" s="30"/>
+      <c r="S1" s="30"/>
+      <c r="T1" s="30"/>
+      <c r="U1" s="30"/>
+      <c r="V1" s="30"/>
+      <c r="W1" s="30"/>
+      <c r="X1" s="30"/>
+      <c r="Y1" s="30"/>
+      <c r="Z1" s="30"/>
+      <c r="AA1" s="30"/>
     </row>
     <row r="2" spans="1:27" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="25" t="s">
-        <v>134</v>
-      </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
-      <c r="L2" s="24"/>
-      <c r="M2" s="24"/>
-      <c r="N2" s="24"/>
-      <c r="O2" s="24"/>
-      <c r="P2" s="24"/>
-      <c r="Q2" s="24"/>
-      <c r="R2" s="24"/>
-      <c r="S2" s="24"/>
-      <c r="T2" s="24"/>
-      <c r="U2" s="24"/>
-      <c r="V2" s="24"/>
-      <c r="W2" s="24"/>
-      <c r="X2" s="24"/>
-      <c r="Y2" s="24"/>
-      <c r="Z2" s="24"/>
-      <c r="AA2" s="24"/>
+      <c r="B2" s="33" t="s">
+        <v>186</v>
+      </c>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
+      <c r="M2" s="30"/>
+      <c r="N2" s="30"/>
+      <c r="O2" s="30"/>
+      <c r="P2" s="30"/>
+      <c r="Q2" s="30"/>
+      <c r="R2" s="30"/>
+      <c r="S2" s="30"/>
+      <c r="T2" s="30"/>
+      <c r="U2" s="30"/>
+      <c r="V2" s="30"/>
+      <c r="W2" s="30"/>
+      <c r="X2" s="30"/>
+      <c r="Y2" s="30"/>
+      <c r="Z2" s="30"/>
+      <c r="AA2" s="30"/>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>135</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5" spans="1:27" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>136</v>
+        <v>188</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>137</v>
+        <v>189</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>138</v>
+        <v>190</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>139</v>
+        <v>191</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>140</v>
+        <v>192</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>141</v>
+        <v>193</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>142</v>
+        <v>194</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>143</v>
+        <v>195</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>144</v>
+        <v>196</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>145</v>
+        <v>197</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>147</v>
+        <v>199</v>
       </c>
       <c r="M5" s="10" t="s">
-        <v>148</v>
+        <v>200</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>149</v>
+        <v>201</v>
       </c>
       <c r="O5" s="10" t="s">
-        <v>150</v>
+        <v>202</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>151</v>
+        <v>203</v>
       </c>
       <c r="Q5" s="10" t="s">
-        <v>152</v>
+        <v>204</v>
       </c>
       <c r="R5" s="10" t="s">
-        <v>153</v>
+        <v>205</v>
       </c>
       <c r="S5" s="10" t="s">
-        <v>154</v>
+        <v>206</v>
       </c>
       <c r="T5" s="10" t="s">
-        <v>155</v>
+        <v>207</v>
       </c>
       <c r="U5" s="10" t="s">
-        <v>156</v>
+        <v>208</v>
       </c>
       <c r="V5" s="10" t="s">
-        <v>157</v>
+        <v>209</v>
       </c>
       <c r="W5" s="10" t="s">
-        <v>158</v>
+        <v>210</v>
       </c>
       <c r="X5" s="10" t="s">
-        <v>159</v>
+        <v>211</v>
       </c>
       <c r="Y5" s="10" t="s">
-        <v>160</v>
+        <v>212</v>
       </c>
       <c r="Z5" s="10" t="s">
-        <v>161</v>
+        <v>213</v>
       </c>
       <c r="AA5" s="10" t="s">
-        <v>162</v>
+        <v>214</v>
       </c>
     </row>
     <row r="6" spans="1:27" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>163</v>
+        <v>215</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>164</v>
+        <v>216</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>165</v>
+        <v>217</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>166</v>
+        <v>218</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>167</v>
+        <v>219</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>168</v>
+        <v>220</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>169</v>
+        <v>221</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>170</v>
+        <v>222</v>
       </c>
       <c r="I6" s="11">
         <v>2</v>
       </c>
       <c r="J6" s="11" t="s">
-        <v>171</v>
+        <v>223</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>172</v>
-      </c>
-      <c r="L6" s="18">
+        <v>224</v>
+      </c>
+      <c r="L6" s="24">
         <v>0.75</v>
       </c>
       <c r="M6" s="11" t="s">
-        <v>173</v>
+        <v>225</v>
       </c>
       <c r="N6" s="11"/>
       <c r="O6" s="11">
         <v>0</v>
       </c>
       <c r="P6" s="11" t="s">
-        <v>174</v>
+        <v>226</v>
       </c>
       <c r="Q6" s="11" t="s">
-        <v>175</v>
+        <v>227</v>
       </c>
       <c r="R6" s="11" t="s">
-        <v>176</v>
+        <v>228</v>
       </c>
       <c r="S6" s="11">
         <v>1</v>
@@ -6660,7 +7161,7 @@
       <c r="Y6" s="11"/>
       <c r="Z6" s="11"/>
       <c r="AA6" s="11" t="s">
-        <v>177</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7" spans="1:27" ht="26.4" x14ac:dyDescent="0.3">
@@ -6668,61 +7169,61 @@
         <f t="shared" ref="A7:A38" si="0">IF(B7="","","SLA-"&amp;TEXT(ROW()-5,"00"))</f>
         <v>SLA-02</v>
       </c>
-      <c r="B7" s="19" t="s">
-        <v>178</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>179</v>
-      </c>
-      <c r="D7" s="19" t="s">
-        <v>166</v>
-      </c>
-      <c r="E7" s="19" t="s">
-        <v>167</v>
-      </c>
-      <c r="F7" s="19" t="s">
-        <v>180</v>
-      </c>
-      <c r="G7" s="19" t="s">
-        <v>181</v>
-      </c>
-      <c r="H7" s="19" t="s">
-        <v>170</v>
-      </c>
-      <c r="I7" s="19">
+      <c r="B7" s="25" t="s">
+        <v>230</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>231</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>218</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>219</v>
+      </c>
+      <c r="F7" s="25" t="s">
+        <v>232</v>
+      </c>
+      <c r="G7" s="25" t="s">
+        <v>233</v>
+      </c>
+      <c r="H7" s="25" t="s">
+        <v>222</v>
+      </c>
+      <c r="I7" s="25">
         <v>2</v>
       </c>
-      <c r="J7" s="19" t="s">
-        <v>171</v>
-      </c>
-      <c r="K7" s="19" t="s">
-        <v>172</v>
-      </c>
-      <c r="L7" s="20"/>
-      <c r="M7" s="19"/>
-      <c r="N7" s="19"/>
-      <c r="O7" s="19">
+      <c r="J7" s="25" t="s">
+        <v>223</v>
+      </c>
+      <c r="K7" s="25" t="s">
+        <v>224</v>
+      </c>
+      <c r="L7" s="26"/>
+      <c r="M7" s="25"/>
+      <c r="N7" s="25"/>
+      <c r="O7" s="25">
         <v>0</v>
       </c>
-      <c r="P7" s="19" t="s">
-        <v>174</v>
-      </c>
-      <c r="Q7" s="19" t="s">
-        <v>175</v>
-      </c>
-      <c r="R7" s="19" t="s">
-        <v>176</v>
-      </c>
-      <c r="S7" s="19"/>
-      <c r="T7" s="19"/>
-      <c r="U7" s="19"/>
-      <c r="V7" s="19"/>
-      <c r="W7" s="19"/>
-      <c r="X7" s="19"/>
-      <c r="Y7" s="19"/>
-      <c r="Z7" s="19"/>
-      <c r="AA7" s="19" t="s">
-        <v>182</v>
+      <c r="P7" s="25" t="s">
+        <v>226</v>
+      </c>
+      <c r="Q7" s="25" t="s">
+        <v>227</v>
+      </c>
+      <c r="R7" s="25" t="s">
+        <v>228</v>
+      </c>
+      <c r="S7" s="25"/>
+      <c r="T7" s="25"/>
+      <c r="U7" s="25"/>
+      <c r="V7" s="25"/>
+      <c r="W7" s="25"/>
+      <c r="X7" s="25"/>
+      <c r="Y7" s="25"/>
+      <c r="Z7" s="25"/>
+      <c r="AA7" s="25" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
@@ -6740,7 +7241,7 @@
       <c r="I8" s="14"/>
       <c r="J8" s="14"/>
       <c r="K8" s="14"/>
-      <c r="L8" s="21"/>
+      <c r="L8" s="27"/>
       <c r="M8" s="14"/>
       <c r="N8" s="14"/>
       <c r="O8" s="14"/>
@@ -6772,7 +7273,7 @@
       <c r="I9" s="14"/>
       <c r="J9" s="14"/>
       <c r="K9" s="14"/>
-      <c r="L9" s="21"/>
+      <c r="L9" s="27"/>
       <c r="M9" s="14"/>
       <c r="N9" s="14"/>
       <c r="O9" s="14"/>
@@ -6804,7 +7305,7 @@
       <c r="I10" s="14"/>
       <c r="J10" s="14"/>
       <c r="K10" s="14"/>
-      <c r="L10" s="21"/>
+      <c r="L10" s="27"/>
       <c r="M10" s="14"/>
       <c r="N10" s="14"/>
       <c r="O10" s="14"/>
@@ -6836,7 +7337,7 @@
       <c r="I11" s="14"/>
       <c r="J11" s="14"/>
       <c r="K11" s="14"/>
-      <c r="L11" s="21"/>
+      <c r="L11" s="27"/>
       <c r="M11" s="14"/>
       <c r="N11" s="14"/>
       <c r="O11" s="14"/>
@@ -6868,7 +7369,7 @@
       <c r="I12" s="14"/>
       <c r="J12" s="14"/>
       <c r="K12" s="14"/>
-      <c r="L12" s="21"/>
+      <c r="L12" s="27"/>
       <c r="M12" s="14"/>
       <c r="N12" s="14"/>
       <c r="O12" s="14"/>
@@ -6900,7 +7401,7 @@
       <c r="I13" s="14"/>
       <c r="J13" s="14"/>
       <c r="K13" s="14"/>
-      <c r="L13" s="21"/>
+      <c r="L13" s="27"/>
       <c r="M13" s="14"/>
       <c r="N13" s="14"/>
       <c r="O13" s="14"/>
@@ -6932,7 +7433,7 @@
       <c r="I14" s="14"/>
       <c r="J14" s="14"/>
       <c r="K14" s="14"/>
-      <c r="L14" s="21"/>
+      <c r="L14" s="27"/>
       <c r="M14" s="14"/>
       <c r="N14" s="14"/>
       <c r="O14" s="14"/>
@@ -6964,7 +7465,7 @@
       <c r="I15" s="14"/>
       <c r="J15" s="14"/>
       <c r="K15" s="14"/>
-      <c r="L15" s="21"/>
+      <c r="L15" s="27"/>
       <c r="M15" s="14"/>
       <c r="N15" s="14"/>
       <c r="O15" s="14"/>
@@ -6996,7 +7497,7 @@
       <c r="I16" s="14"/>
       <c r="J16" s="14"/>
       <c r="K16" s="14"/>
-      <c r="L16" s="21"/>
+      <c r="L16" s="27"/>
       <c r="M16" s="14"/>
       <c r="N16" s="14"/>
       <c r="O16" s="14"/>
@@ -7028,7 +7529,7 @@
       <c r="I17" s="14"/>
       <c r="J17" s="14"/>
       <c r="K17" s="14"/>
-      <c r="L17" s="21"/>
+      <c r="L17" s="27"/>
       <c r="M17" s="14"/>
       <c r="N17" s="14"/>
       <c r="O17" s="14"/>
@@ -7060,7 +7561,7 @@
       <c r="I18" s="14"/>
       <c r="J18" s="14"/>
       <c r="K18" s="14"/>
-      <c r="L18" s="21"/>
+      <c r="L18" s="27"/>
       <c r="M18" s="14"/>
       <c r="N18" s="14"/>
       <c r="O18" s="14"/>
@@ -7092,7 +7593,7 @@
       <c r="I19" s="14"/>
       <c r="J19" s="14"/>
       <c r="K19" s="14"/>
-      <c r="L19" s="21"/>
+      <c r="L19" s="27"/>
       <c r="M19" s="14"/>
       <c r="N19" s="14"/>
       <c r="O19" s="14"/>
@@ -7124,7 +7625,7 @@
       <c r="I20" s="14"/>
       <c r="J20" s="14"/>
       <c r="K20" s="14"/>
-      <c r="L20" s="21"/>
+      <c r="L20" s="27"/>
       <c r="M20" s="14"/>
       <c r="N20" s="14"/>
       <c r="O20" s="14"/>
@@ -7156,7 +7657,7 @@
       <c r="I21" s="14"/>
       <c r="J21" s="14"/>
       <c r="K21" s="14"/>
-      <c r="L21" s="21"/>
+      <c r="L21" s="27"/>
       <c r="M21" s="14"/>
       <c r="N21" s="14"/>
       <c r="O21" s="14"/>
@@ -7188,7 +7689,7 @@
       <c r="I22" s="14"/>
       <c r="J22" s="14"/>
       <c r="K22" s="14"/>
-      <c r="L22" s="21"/>
+      <c r="L22" s="27"/>
       <c r="M22" s="14"/>
       <c r="N22" s="14"/>
       <c r="O22" s="14"/>
@@ -7220,7 +7721,7 @@
       <c r="I23" s="14"/>
       <c r="J23" s="14"/>
       <c r="K23" s="14"/>
-      <c r="L23" s="21"/>
+      <c r="L23" s="27"/>
       <c r="M23" s="14"/>
       <c r="N23" s="14"/>
       <c r="O23" s="14"/>
@@ -7252,7 +7753,7 @@
       <c r="I24" s="14"/>
       <c r="J24" s="14"/>
       <c r="K24" s="14"/>
-      <c r="L24" s="21"/>
+      <c r="L24" s="27"/>
       <c r="M24" s="14"/>
       <c r="N24" s="14"/>
       <c r="O24" s="14"/>
@@ -7284,7 +7785,7 @@
       <c r="I25" s="14"/>
       <c r="J25" s="14"/>
       <c r="K25" s="14"/>
-      <c r="L25" s="21"/>
+      <c r="L25" s="27"/>
       <c r="M25" s="14"/>
       <c r="N25" s="14"/>
       <c r="O25" s="14"/>
@@ -7316,7 +7817,7 @@
       <c r="I26" s="14"/>
       <c r="J26" s="14"/>
       <c r="K26" s="14"/>
-      <c r="L26" s="21"/>
+      <c r="L26" s="27"/>
       <c r="M26" s="14"/>
       <c r="N26" s="14"/>
       <c r="O26" s="14"/>
@@ -7348,7 +7849,7 @@
       <c r="I27" s="14"/>
       <c r="J27" s="14"/>
       <c r="K27" s="14"/>
-      <c r="L27" s="21"/>
+      <c r="L27" s="27"/>
       <c r="M27" s="14"/>
       <c r="N27" s="14"/>
       <c r="O27" s="14"/>
@@ -7380,7 +7881,7 @@
       <c r="I28" s="14"/>
       <c r="J28" s="14"/>
       <c r="K28" s="14"/>
-      <c r="L28" s="21"/>
+      <c r="L28" s="27"/>
       <c r="M28" s="14"/>
       <c r="N28" s="14"/>
       <c r="O28" s="14"/>
@@ -7412,7 +7913,7 @@
       <c r="I29" s="14"/>
       <c r="J29" s="14"/>
       <c r="K29" s="14"/>
-      <c r="L29" s="21"/>
+      <c r="L29" s="27"/>
       <c r="M29" s="14"/>
       <c r="N29" s="14"/>
       <c r="O29" s="14"/>
@@ -7444,7 +7945,7 @@
       <c r="I30" s="14"/>
       <c r="J30" s="14"/>
       <c r="K30" s="14"/>
-      <c r="L30" s="21"/>
+      <c r="L30" s="27"/>
       <c r="M30" s="14"/>
       <c r="N30" s="14"/>
       <c r="O30" s="14"/>
@@ -7476,7 +7977,7 @@
       <c r="I31" s="14"/>
       <c r="J31" s="14"/>
       <c r="K31" s="14"/>
-      <c r="L31" s="21"/>
+      <c r="L31" s="27"/>
       <c r="M31" s="14"/>
       <c r="N31" s="14"/>
       <c r="O31" s="14"/>
@@ -7508,7 +8009,7 @@
       <c r="I32" s="14"/>
       <c r="J32" s="14"/>
       <c r="K32" s="14"/>
-      <c r="L32" s="21"/>
+      <c r="L32" s="27"/>
       <c r="M32" s="14"/>
       <c r="N32" s="14"/>
       <c r="O32" s="14"/>
@@ -7540,7 +8041,7 @@
       <c r="I33" s="14"/>
       <c r="J33" s="14"/>
       <c r="K33" s="14"/>
-      <c r="L33" s="21"/>
+      <c r="L33" s="27"/>
       <c r="M33" s="14"/>
       <c r="N33" s="14"/>
       <c r="O33" s="14"/>
@@ -7572,7 +8073,7 @@
       <c r="I34" s="14"/>
       <c r="J34" s="14"/>
       <c r="K34" s="14"/>
-      <c r="L34" s="21"/>
+      <c r="L34" s="27"/>
       <c r="M34" s="14"/>
       <c r="N34" s="14"/>
       <c r="O34" s="14"/>
@@ -7604,7 +8105,7 @@
       <c r="I35" s="14"/>
       <c r="J35" s="14"/>
       <c r="K35" s="14"/>
-      <c r="L35" s="21"/>
+      <c r="L35" s="27"/>
       <c r="M35" s="14"/>
       <c r="N35" s="14"/>
       <c r="O35" s="14"/>
@@ -7636,7 +8137,7 @@
       <c r="I36" s="14"/>
       <c r="J36" s="14"/>
       <c r="K36" s="14"/>
-      <c r="L36" s="21"/>
+      <c r="L36" s="27"/>
       <c r="M36" s="14"/>
       <c r="N36" s="14"/>
       <c r="O36" s="14"/>
@@ -7668,7 +8169,7 @@
       <c r="I37" s="14"/>
       <c r="J37" s="14"/>
       <c r="K37" s="14"/>
-      <c r="L37" s="21"/>
+      <c r="L37" s="27"/>
       <c r="M37" s="14"/>
       <c r="N37" s="14"/>
       <c r="O37" s="14"/>
@@ -7700,7 +8201,7 @@
       <c r="I38" s="14"/>
       <c r="J38" s="14"/>
       <c r="K38" s="14"/>
-      <c r="L38" s="21"/>
+      <c r="L38" s="27"/>
       <c r="M38" s="14"/>
       <c r="N38" s="14"/>
       <c r="O38" s="14"/>
@@ -7732,7 +8233,7 @@
       <c r="I39" s="14"/>
       <c r="J39" s="14"/>
       <c r="K39" s="14"/>
-      <c r="L39" s="21"/>
+      <c r="L39" s="27"/>
       <c r="M39" s="14"/>
       <c r="N39" s="14"/>
       <c r="O39" s="14"/>
@@ -7764,7 +8265,7 @@
       <c r="I40" s="14"/>
       <c r="J40" s="14"/>
       <c r="K40" s="14"/>
-      <c r="L40" s="21"/>
+      <c r="L40" s="27"/>
       <c r="M40" s="14"/>
       <c r="N40" s="14"/>
       <c r="O40" s="14"/>
@@ -7796,7 +8297,7 @@
       <c r="I41" s="14"/>
       <c r="J41" s="14"/>
       <c r="K41" s="14"/>
-      <c r="L41" s="21"/>
+      <c r="L41" s="27"/>
       <c r="M41" s="14"/>
       <c r="N41" s="14"/>
       <c r="O41" s="14"/>
@@ -7828,7 +8329,7 @@
       <c r="I42" s="14"/>
       <c r="J42" s="14"/>
       <c r="K42" s="14"/>
-      <c r="L42" s="21"/>
+      <c r="L42" s="27"/>
       <c r="M42" s="14"/>
       <c r="N42" s="14"/>
       <c r="O42" s="14"/>
@@ -7860,7 +8361,7 @@
       <c r="I43" s="14"/>
       <c r="J43" s="14"/>
       <c r="K43" s="14"/>
-      <c r="L43" s="21"/>
+      <c r="L43" s="27"/>
       <c r="M43" s="14"/>
       <c r="N43" s="14"/>
       <c r="O43" s="14"/>
@@ -7892,7 +8393,7 @@
       <c r="I44" s="14"/>
       <c r="J44" s="14"/>
       <c r="K44" s="14"/>
-      <c r="L44" s="21"/>
+      <c r="L44" s="27"/>
       <c r="M44" s="14"/>
       <c r="N44" s="14"/>
       <c r="O44" s="14"/>
@@ -7924,7 +8425,7 @@
       <c r="I45" s="14"/>
       <c r="J45" s="14"/>
       <c r="K45" s="14"/>
-      <c r="L45" s="21"/>
+      <c r="L45" s="27"/>
       <c r="M45" s="14"/>
       <c r="N45" s="14"/>
       <c r="O45" s="14"/>
@@ -7956,7 +8457,7 @@
       <c r="I46" s="14"/>
       <c r="J46" s="14"/>
       <c r="K46" s="14"/>
-      <c r="L46" s="21"/>
+      <c r="L46" s="27"/>
       <c r="M46" s="14"/>
       <c r="N46" s="14"/>
       <c r="O46" s="14"/>
@@ -7988,7 +8489,7 @@
       <c r="I47" s="14"/>
       <c r="J47" s="14"/>
       <c r="K47" s="14"/>
-      <c r="L47" s="21"/>
+      <c r="L47" s="27"/>
       <c r="M47" s="14"/>
       <c r="N47" s="14"/>
       <c r="O47" s="14"/>
@@ -8020,7 +8521,7 @@
       <c r="I48" s="14"/>
       <c r="J48" s="14"/>
       <c r="K48" s="14"/>
-      <c r="L48" s="21"/>
+      <c r="L48" s="27"/>
       <c r="M48" s="14"/>
       <c r="N48" s="14"/>
       <c r="O48" s="14"/>
@@ -8052,7 +8553,7 @@
       <c r="I49" s="14"/>
       <c r="J49" s="14"/>
       <c r="K49" s="14"/>
-      <c r="L49" s="21"/>
+      <c r="L49" s="27"/>
       <c r="M49" s="14"/>
       <c r="N49" s="14"/>
       <c r="O49" s="14"/>
@@ -8084,7 +8585,7 @@
       <c r="I50" s="14"/>
       <c r="J50" s="14"/>
       <c r="K50" s="14"/>
-      <c r="L50" s="21"/>
+      <c r="L50" s="27"/>
       <c r="M50" s="14"/>
       <c r="N50" s="14"/>
       <c r="O50" s="14"/>
@@ -8116,7 +8617,7 @@
       <c r="I51" s="14"/>
       <c r="J51" s="14"/>
       <c r="K51" s="14"/>
-      <c r="L51" s="21"/>
+      <c r="L51" s="27"/>
       <c r="M51" s="14"/>
       <c r="N51" s="14"/>
       <c r="O51" s="14"/>
@@ -8148,7 +8649,7 @@
       <c r="I52" s="14"/>
       <c r="J52" s="14"/>
       <c r="K52" s="14"/>
-      <c r="L52" s="21"/>
+      <c r="L52" s="27"/>
       <c r="M52" s="14"/>
       <c r="N52" s="14"/>
       <c r="O52" s="14"/>
@@ -8180,7 +8681,7 @@
       <c r="I53" s="14"/>
       <c r="J53" s="14"/>
       <c r="K53" s="14"/>
-      <c r="L53" s="21"/>
+      <c r="L53" s="27"/>
       <c r="M53" s="14"/>
       <c r="N53" s="14"/>
       <c r="O53" s="14"/>
@@ -8212,7 +8713,7 @@
       <c r="I54" s="14"/>
       <c r="J54" s="14"/>
       <c r="K54" s="14"/>
-      <c r="L54" s="21"/>
+      <c r="L54" s="27"/>
       <c r="M54" s="14"/>
       <c r="N54" s="14"/>
       <c r="O54" s="14"/>
@@ -8244,7 +8745,7 @@
       <c r="I55" s="14"/>
       <c r="J55" s="14"/>
       <c r="K55" s="14"/>
-      <c r="L55" s="21"/>
+      <c r="L55" s="27"/>
       <c r="M55" s="14"/>
       <c r="N55" s="14"/>
       <c r="O55" s="14"/>
@@ -8276,7 +8777,7 @@
       <c r="I56" s="14"/>
       <c r="J56" s="14"/>
       <c r="K56" s="14"/>
-      <c r="L56" s="21"/>
+      <c r="L56" s="27"/>
       <c r="M56" s="14"/>
       <c r="N56" s="14"/>
       <c r="O56" s="14"/>
@@ -8308,7 +8809,7 @@
       <c r="I57" s="14"/>
       <c r="J57" s="14"/>
       <c r="K57" s="14"/>
-      <c r="L57" s="21"/>
+      <c r="L57" s="27"/>
       <c r="M57" s="14"/>
       <c r="N57" s="14"/>
       <c r="O57" s="14"/>
@@ -8340,7 +8841,7 @@
       <c r="I58" s="14"/>
       <c r="J58" s="14"/>
       <c r="K58" s="14"/>
-      <c r="L58" s="21"/>
+      <c r="L58" s="27"/>
       <c r="M58" s="14"/>
       <c r="N58" s="14"/>
       <c r="O58" s="14"/>
@@ -8372,7 +8873,7 @@
       <c r="I59" s="14"/>
       <c r="J59" s="14"/>
       <c r="K59" s="14"/>
-      <c r="L59" s="21"/>
+      <c r="L59" s="27"/>
       <c r="M59" s="14"/>
       <c r="N59" s="14"/>
       <c r="O59" s="14"/>
@@ -8404,7 +8905,7 @@
       <c r="I60" s="14"/>
       <c r="J60" s="14"/>
       <c r="K60" s="14"/>
-      <c r="L60" s="21"/>
+      <c r="L60" s="27"/>
       <c r="M60" s="14"/>
       <c r="N60" s="14"/>
       <c r="O60" s="14"/>
@@ -8436,7 +8937,7 @@
       <c r="I61" s="14"/>
       <c r="J61" s="14"/>
       <c r="K61" s="14"/>
-      <c r="L61" s="21"/>
+      <c r="L61" s="27"/>
       <c r="M61" s="14"/>
       <c r="N61" s="14"/>
       <c r="O61" s="14"/>
@@ -8468,7 +8969,7 @@
       <c r="I62" s="14"/>
       <c r="J62" s="14"/>
       <c r="K62" s="14"/>
-      <c r="L62" s="21"/>
+      <c r="L62" s="27"/>
       <c r="M62" s="14"/>
       <c r="N62" s="14"/>
       <c r="O62" s="14"/>
@@ -8500,7 +9001,7 @@
       <c r="I63" s="14"/>
       <c r="J63" s="14"/>
       <c r="K63" s="14"/>
-      <c r="L63" s="21"/>
+      <c r="L63" s="27"/>
       <c r="M63" s="14"/>
       <c r="N63" s="14"/>
       <c r="O63" s="14"/>
@@ -8532,7 +9033,7 @@
       <c r="I64" s="14"/>
       <c r="J64" s="14"/>
       <c r="K64" s="14"/>
-      <c r="L64" s="21"/>
+      <c r="L64" s="27"/>
       <c r="M64" s="14"/>
       <c r="N64" s="14"/>
       <c r="O64" s="14"/>
@@ -8564,7 +9065,7 @@
       <c r="I65" s="14"/>
       <c r="J65" s="14"/>
       <c r="K65" s="14"/>
-      <c r="L65" s="21"/>
+      <c r="L65" s="27"/>
       <c r="M65" s="14"/>
       <c r="N65" s="14"/>
       <c r="O65" s="14"/>
@@ -8596,7 +9097,7 @@
       <c r="I66" s="14"/>
       <c r="J66" s="14"/>
       <c r="K66" s="14"/>
-      <c r="L66" s="21"/>
+      <c r="L66" s="27"/>
       <c r="M66" s="14"/>
       <c r="N66" s="14"/>
       <c r="O66" s="14"/>
@@ -8681,7 +9182,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF36B78E"/>
@@ -8699,90 +9200,90 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="23" t="s">
-        <v>183</v>
-      </c>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
+      <c r="B1" s="29" t="s">
+        <v>235</v>
+      </c>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
     </row>
     <row r="2" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="25" t="s">
-        <v>184</v>
-      </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="B2" s="33" t="s">
+        <v>236</v>
+      </c>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>185</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>186</v>
+        <v>238</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>187</v>
+        <v>239</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>188</v>
+        <v>240</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>189</v>
+        <v>241</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>190</v>
+        <v>242</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>191</v>
+        <v>243</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>192</v>
+        <v>244</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>162</v>
+        <v>214</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>173</v>
+        <v>225</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>193</v>
+        <v>245</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>194</v>
+        <v>246</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>195</v>
+        <v>247</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>196</v>
+        <v>248</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>197</v>
+        <v>249</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>198</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A7" s="14" t="s">
-        <v>173</v>
+        <v>225</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>199</v>
+        <v>251</v>
       </c>
       <c r="C7" s="14"/>
       <c r="D7" s="14"/>
@@ -8793,10 +9294,10 @@
     </row>
     <row r="8" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
-        <v>200</v>
+        <v>252</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>201</v>
+        <v>253</v>
       </c>
       <c r="C8" s="14"/>
       <c r="D8" s="14"/>
@@ -8807,10 +9308,10 @@
     </row>
     <row r="9" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A9" s="14" t="s">
-        <v>202</v>
+        <v>254</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>203</v>
+        <v>255</v>
       </c>
       <c r="C9" s="14"/>
       <c r="D9" s="14"/>
@@ -8821,10 +9322,10 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
-        <v>204</v>
+        <v>256</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>205</v>
+        <v>257</v>
       </c>
       <c r="C10" s="14"/>
       <c r="D10" s="14"/>
@@ -8835,10 +9336,10 @@
     </row>
     <row r="11" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
-        <v>206</v>
+        <v>258</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>207</v>
+        <v>259</v>
       </c>
       <c r="C11" s="14"/>
       <c r="D11" s="14"/>
@@ -8849,10 +9350,10 @@
     </row>
     <row r="12" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A12" s="14" t="s">
-        <v>208</v>
+        <v>260</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>209</v>
+        <v>261</v>
       </c>
       <c r="C12" s="14"/>
       <c r="D12" s="14"/>
@@ -8863,10 +9364,10 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="14" t="s">
-        <v>174</v>
+        <v>226</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>210</v>
+        <v>262</v>
       </c>
       <c r="C13" s="14"/>
       <c r="D13" s="14"/>
@@ -8877,10 +9378,10 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="14" t="s">
-        <v>211</v>
+        <v>263</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>212</v>
+        <v>264</v>
       </c>
       <c r="C14" s="14"/>
       <c r="D14" s="14"/>
@@ -9433,380 +9934,380 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A1" s="22" t="s">
-        <v>93</v>
-      </c>
-      <c r="B1" s="22" t="s">
-        <v>97</v>
-      </c>
-      <c r="C1" s="22" t="s">
-        <v>213</v>
-      </c>
-      <c r="D1" s="22" t="s">
-        <v>214</v>
-      </c>
-      <c r="E1" s="22" t="s">
-        <v>140</v>
-      </c>
-      <c r="F1" s="22" t="s">
-        <v>215</v>
-      </c>
-      <c r="G1" s="22" t="s">
-        <v>145</v>
-      </c>
-      <c r="H1" s="22" t="s">
-        <v>146</v>
-      </c>
-      <c r="I1" s="22" t="s">
-        <v>216</v>
-      </c>
-      <c r="J1" s="22" t="s">
-        <v>217</v>
-      </c>
-      <c r="K1" s="22" t="s">
-        <v>218</v>
-      </c>
-      <c r="L1" s="22" t="s">
-        <v>219</v>
-      </c>
-      <c r="M1" s="22" t="s">
-        <v>220</v>
-      </c>
-      <c r="N1" s="22" t="s">
-        <v>221</v>
-      </c>
-      <c r="O1" s="22" t="s">
-        <v>222</v>
+      <c r="A1" s="28" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1" s="28" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1" s="28" t="s">
+        <v>265</v>
+      </c>
+      <c r="D1" s="28" t="s">
+        <v>266</v>
+      </c>
+      <c r="E1" s="28" t="s">
+        <v>192</v>
+      </c>
+      <c r="F1" s="28" t="s">
+        <v>267</v>
+      </c>
+      <c r="G1" s="28" t="s">
+        <v>197</v>
+      </c>
+      <c r="H1" s="28" t="s">
+        <v>198</v>
+      </c>
+      <c r="I1" s="28" t="s">
+        <v>268</v>
+      </c>
+      <c r="J1" s="28" t="s">
+        <v>269</v>
+      </c>
+      <c r="K1" s="28" t="s">
+        <v>270</v>
+      </c>
+      <c r="L1" s="28" t="s">
+        <v>271</v>
+      </c>
+      <c r="M1" s="28" t="s">
+        <v>272</v>
+      </c>
+      <c r="N1" s="28" t="s">
+        <v>273</v>
+      </c>
+      <c r="O1" s="28" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D2" t="s">
-        <v>166</v>
+        <v>218</v>
       </c>
       <c r="E2" t="s">
-        <v>167</v>
+        <v>219</v>
       </c>
       <c r="F2" t="s">
-        <v>165</v>
+        <v>217</v>
       </c>
       <c r="G2" t="s">
-        <v>223</v>
+        <v>275</v>
       </c>
       <c r="H2" t="s">
-        <v>172</v>
+        <v>224</v>
       </c>
       <c r="I2" t="s">
-        <v>176</v>
+        <v>228</v>
       </c>
       <c r="J2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="K2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="L2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="M2" t="s">
-        <v>224</v>
+        <v>276</v>
       </c>
       <c r="N2" t="s">
+        <v>277</v>
+      </c>
+      <c r="O2" t="s">
         <v>225</v>
-      </c>
-      <c r="O2" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>226</v>
+        <v>169</v>
       </c>
       <c r="B3" t="s">
-        <v>227</v>
+        <v>278</v>
       </c>
       <c r="C3" t="s">
-        <v>228</v>
+        <v>279</v>
       </c>
       <c r="D3" t="s">
-        <v>229</v>
+        <v>280</v>
       </c>
       <c r="E3" t="s">
-        <v>230</v>
+        <v>281</v>
       </c>
       <c r="F3" t="s">
-        <v>179</v>
+        <v>231</v>
       </c>
       <c r="G3" t="s">
-        <v>171</v>
+        <v>223</v>
       </c>
       <c r="H3" t="s">
-        <v>231</v>
+        <v>282</v>
       </c>
       <c r="I3" t="s">
-        <v>232</v>
+        <v>283</v>
       </c>
       <c r="J3" t="s">
-        <v>197</v>
+        <v>249</v>
       </c>
       <c r="K3" t="s">
-        <v>233</v>
+        <v>284</v>
       </c>
       <c r="L3" t="s">
-        <v>234</v>
+        <v>285</v>
       </c>
       <c r="M3" t="s">
-        <v>235</v>
+        <v>286</v>
       </c>
       <c r="N3" t="s">
-        <v>236</v>
+        <v>287</v>
       </c>
       <c r="O3" t="s">
-        <v>200</v>
+        <v>252</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>237</v>
+        <v>135</v>
       </c>
       <c r="B4" t="s">
-        <v>238</v>
+        <v>288</v>
       </c>
       <c r="C4" t="s">
-        <v>239</v>
+        <v>289</v>
       </c>
       <c r="D4" t="s">
-        <v>240</v>
+        <v>290</v>
       </c>
       <c r="E4" t="s">
-        <v>241</v>
+        <v>291</v>
       </c>
       <c r="F4" t="s">
-        <v>242</v>
+        <v>292</v>
       </c>
       <c r="G4" t="s">
-        <v>243</v>
+        <v>293</v>
       </c>
       <c r="I4" t="s">
-        <v>244</v>
+        <v>294</v>
       </c>
       <c r="K4" t="s">
-        <v>245</v>
+        <v>295</v>
       </c>
       <c r="M4" t="s">
-        <v>246</v>
+        <v>296</v>
       </c>
       <c r="N4" t="s">
-        <v>247</v>
+        <v>297</v>
       </c>
       <c r="O4" t="s">
-        <v>202</v>
+        <v>254</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>248</v>
+        <v>298</v>
       </c>
       <c r="B5" t="s">
-        <v>249</v>
+        <v>299</v>
       </c>
       <c r="C5" t="s">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="D5" t="s">
-        <v>251</v>
+        <v>301</v>
       </c>
       <c r="E5" t="s">
-        <v>252</v>
+        <v>302</v>
       </c>
       <c r="F5" t="s">
-        <v>253</v>
+        <v>303</v>
       </c>
       <c r="G5" t="s">
-        <v>254</v>
+        <v>304</v>
       </c>
       <c r="I5" t="s">
-        <v>255</v>
+        <v>305</v>
       </c>
       <c r="K5" t="s">
+        <v>306</v>
+      </c>
+      <c r="M5" t="s">
+        <v>307</v>
+      </c>
+      <c r="N5" t="s">
+        <v>308</v>
+      </c>
+      <c r="O5" t="s">
         <v>256</v>
-      </c>
-      <c r="M5" t="s">
-        <v>257</v>
-      </c>
-      <c r="N5" t="s">
-        <v>258</v>
-      </c>
-      <c r="O5" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D6" t="s">
-        <v>259</v>
+        <v>309</v>
       </c>
       <c r="E6" t="s">
-        <v>260</v>
+        <v>310</v>
       </c>
       <c r="F6" t="s">
-        <v>261</v>
+        <v>311</v>
       </c>
       <c r="K6" t="s">
-        <v>262</v>
+        <v>312</v>
       </c>
       <c r="M6" t="s">
-        <v>263</v>
+        <v>313</v>
       </c>
       <c r="N6" t="s">
-        <v>264</v>
+        <v>314</v>
       </c>
       <c r="O6" t="s">
-        <v>206</v>
+        <v>258</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>265</v>
+        <v>315</v>
       </c>
       <c r="D7" t="s">
-        <v>266</v>
+        <v>316</v>
       </c>
       <c r="F7" t="s">
-        <v>267</v>
+        <v>317</v>
       </c>
       <c r="M7" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="N7" t="s">
-        <v>268</v>
+        <v>318</v>
       </c>
       <c r="O7" t="s">
-        <v>208</v>
+        <v>260</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>269</v>
+        <v>319</v>
       </c>
       <c r="D8" t="s">
-        <v>270</v>
+        <v>320</v>
       </c>
       <c r="M8" t="s">
-        <v>271</v>
+        <v>321</v>
       </c>
       <c r="N8" t="s">
-        <v>272</v>
+        <v>322</v>
       </c>
       <c r="O8" t="s">
-        <v>174</v>
+        <v>226</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>273</v>
+        <v>323</v>
       </c>
       <c r="D9" t="s">
-        <v>274</v>
+        <v>324</v>
       </c>
       <c r="M9" t="s">
-        <v>275</v>
+        <v>325</v>
       </c>
       <c r="N9" t="s">
-        <v>275</v>
+        <v>325</v>
       </c>
       <c r="O9" t="s">
-        <v>211</v>
+        <v>263</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>276</v>
+        <v>326</v>
       </c>
       <c r="D10" t="s">
-        <v>277</v>
+        <v>327</v>
       </c>
       <c r="M10" t="s">
-        <v>278</v>
+        <v>328</v>
       </c>
       <c r="N10" t="s">
-        <v>279</v>
+        <v>329</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>267</v>
+        <v>317</v>
       </c>
       <c r="D11" t="s">
-        <v>280</v>
+        <v>330</v>
       </c>
       <c r="M11" t="s">
-        <v>281</v>
+        <v>331</v>
       </c>
       <c r="N11" t="s">
-        <v>282</v>
+        <v>332</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="D12" t="s">
-        <v>267</v>
+        <v>317</v>
       </c>
       <c r="M12" t="s">
-        <v>283</v>
+        <v>333</v>
       </c>
       <c r="N12" t="s">
-        <v>284</v>
+        <v>334</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M13" t="s">
-        <v>285</v>
+        <v>335</v>
       </c>
       <c r="N13" t="s">
-        <v>286</v>
+        <v>336</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M14" t="s">
-        <v>287</v>
+        <v>337</v>
       </c>
       <c r="N14" t="s">
-        <v>288</v>
+        <v>338</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M15" t="s">
-        <v>289</v>
+        <v>339</v>
       </c>
       <c r="N15" t="s">
-        <v>290</v>
+        <v>340</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M16" t="s">
-        <v>291</v>
+        <v>341</v>
       </c>
       <c r="N16" t="s">
-        <v>292</v>
+        <v>342</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
BR-006: reports about Internal Audit stay on the normal workflow
Decision recorded on the impact sheet: no third escalation question.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/WB-Requirements-and-SLA-Template-v1.3.xlsx
+++ b/docs/WB-Requirements-and-SLA-Template-v1.3.xlsx
@@ -345,7 +345,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="344">
   <si>
     <t>Whistleblowing Reporting Portal - Requirements Template</t>
   </si>
@@ -918,6 +918,9 @@
   </si>
   <si>
     <t>Is that acceptable, or is a third question needed?</t>
+  </si>
+  <si>
+    <t>Agreed (21/10/2026): acceptable. A report about Internal Audit follows the normal workflow as built today; no third question.</t>
   </si>
   <si>
     <t>Documentation and training</t>
@@ -1537,7 +1540,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1592,6 +1595,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2151,16 +2157,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:3" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="30"/>
+      <c r="C1" s="31"/>
     </row>
     <row r="2" spans="2:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="30"/>
+      <c r="C2" s="31"/>
     </row>
     <row r="4" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
@@ -2367,10 +2373,10 @@
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B35" s="31" t="s">
+      <c r="B35" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="C35" s="32"/>
+      <c r="C35" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2405,38 +2411,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
-      <c r="M1" s="30"/>
-      <c r="N1" s="30"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="31"/>
+      <c r="M1" s="31"/>
+      <c r="N1" s="31"/>
     </row>
     <row r="2" spans="1:14" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
-      <c r="M2" s="30"/>
-      <c r="N2" s="30"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="31"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -4072,34 +4078,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="31"/>
     </row>
     <row r="2" spans="1:12" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -5433,34 +5439,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="31"/>
     </row>
     <row r="2" spans="1:12" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -6665,22 +6671,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="30" t="s">
         <v>140</v>
       </c>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
     </row>
     <row r="2" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="34" t="s">
         <v>141</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -6851,7 +6857,7 @@
       </c>
       <c r="F13" s="14"/>
     </row>
-    <row r="14" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A14" s="19">
         <v>9</v>
       </c>
@@ -6867,20 +6873,22 @@
       <c r="E14" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="F14" s="14"/>
+      <c r="F14" s="24" t="s">
+        <v>180</v>
+      </c>
     </row>
     <row r="15" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A15" s="21">
         <v>10</v>
       </c>
       <c r="B15" s="22" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C15" s="21" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E15" s="21" t="s">
         <v>66</v>
@@ -6892,13 +6900,13 @@
         <v>11</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C16" s="19" t="s">
         <v>66</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E16" s="19" t="s">
         <v>66</v>
@@ -6950,205 +6958,205 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="29" t="s">
-        <v>185</v>
-      </c>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
-      <c r="M1" s="30"/>
-      <c r="N1" s="30"/>
-      <c r="O1" s="30"/>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="30"/>
-      <c r="R1" s="30"/>
-      <c r="S1" s="30"/>
-      <c r="T1" s="30"/>
-      <c r="U1" s="30"/>
-      <c r="V1" s="30"/>
-      <c r="W1" s="30"/>
-      <c r="X1" s="30"/>
-      <c r="Y1" s="30"/>
-      <c r="Z1" s="30"/>
-      <c r="AA1" s="30"/>
+      <c r="B1" s="30" t="s">
+        <v>186</v>
+      </c>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="31"/>
+      <c r="M1" s="31"/>
+      <c r="N1" s="31"/>
+      <c r="O1" s="31"/>
+      <c r="P1" s="31"/>
+      <c r="Q1" s="31"/>
+      <c r="R1" s="31"/>
+      <c r="S1" s="31"/>
+      <c r="T1" s="31"/>
+      <c r="U1" s="31"/>
+      <c r="V1" s="31"/>
+      <c r="W1" s="31"/>
+      <c r="X1" s="31"/>
+      <c r="Y1" s="31"/>
+      <c r="Z1" s="31"/>
+      <c r="AA1" s="31"/>
     </row>
     <row r="2" spans="1:27" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="33" t="s">
-        <v>186</v>
-      </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
-      <c r="M2" s="30"/>
-      <c r="N2" s="30"/>
-      <c r="O2" s="30"/>
-      <c r="P2" s="30"/>
-      <c r="Q2" s="30"/>
-      <c r="R2" s="30"/>
-      <c r="S2" s="30"/>
-      <c r="T2" s="30"/>
-      <c r="U2" s="30"/>
-      <c r="V2" s="30"/>
-      <c r="W2" s="30"/>
-      <c r="X2" s="30"/>
-      <c r="Y2" s="30"/>
-      <c r="Z2" s="30"/>
-      <c r="AA2" s="30"/>
+      <c r="B2" s="34" t="s">
+        <v>187</v>
+      </c>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="31"/>
+      <c r="O2" s="31"/>
+      <c r="P2" s="31"/>
+      <c r="Q2" s="31"/>
+      <c r="R2" s="31"/>
+      <c r="S2" s="31"/>
+      <c r="T2" s="31"/>
+      <c r="U2" s="31"/>
+      <c r="V2" s="31"/>
+      <c r="W2" s="31"/>
+      <c r="X2" s="31"/>
+      <c r="Y2" s="31"/>
+      <c r="Z2" s="31"/>
+      <c r="AA2" s="31"/>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="5" spans="1:27" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="M5" s="10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="O5" s="10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="Q5" s="10" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="R5" s="10" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="S5" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="T5" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="U5" s="10" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="V5" s="10" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="W5" s="10" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="X5" s="10" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="Y5" s="10" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="Z5" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AA5" s="10" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="6" spans="1:27" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="I6" s="11">
         <v>2</v>
       </c>
       <c r="J6" s="11" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>224</v>
-      </c>
-      <c r="L6" s="24">
+        <v>225</v>
+      </c>
+      <c r="L6" s="25">
         <v>0.75</v>
       </c>
       <c r="M6" s="11" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="N6" s="11"/>
       <c r="O6" s="11">
         <v>0</v>
       </c>
       <c r="P6" s="11" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="Q6" s="11" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="R6" s="11" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="S6" s="11">
         <v>1</v>
@@ -7161,7 +7169,7 @@
       <c r="Y6" s="11"/>
       <c r="Z6" s="11"/>
       <c r="AA6" s="11" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="7" spans="1:27" ht="26.4" x14ac:dyDescent="0.3">
@@ -7169,61 +7177,61 @@
         <f t="shared" ref="A7:A38" si="0">IF(B7="","","SLA-"&amp;TEXT(ROW()-5,"00"))</f>
         <v>SLA-02</v>
       </c>
-      <c r="B7" s="25" t="s">
-        <v>230</v>
-      </c>
-      <c r="C7" s="25" t="s">
+      <c r="B7" s="26" t="s">
         <v>231</v>
       </c>
-      <c r="D7" s="25" t="s">
-        <v>218</v>
-      </c>
-      <c r="E7" s="25" t="s">
+      <c r="C7" s="26" t="s">
+        <v>232</v>
+      </c>
+      <c r="D7" s="26" t="s">
         <v>219</v>
       </c>
-      <c r="F7" s="25" t="s">
-        <v>232</v>
-      </c>
-      <c r="G7" s="25" t="s">
+      <c r="E7" s="26" t="s">
+        <v>220</v>
+      </c>
+      <c r="F7" s="26" t="s">
         <v>233</v>
       </c>
-      <c r="H7" s="25" t="s">
-        <v>222</v>
-      </c>
-      <c r="I7" s="25">
+      <c r="G7" s="26" t="s">
+        <v>234</v>
+      </c>
+      <c r="H7" s="26" t="s">
+        <v>223</v>
+      </c>
+      <c r="I7" s="26">
         <v>2</v>
       </c>
-      <c r="J7" s="25" t="s">
-        <v>223</v>
-      </c>
-      <c r="K7" s="25" t="s">
+      <c r="J7" s="26" t="s">
         <v>224</v>
       </c>
-      <c r="L7" s="26"/>
-      <c r="M7" s="25"/>
-      <c r="N7" s="25"/>
-      <c r="O7" s="25">
+      <c r="K7" s="26" t="s">
+        <v>225</v>
+      </c>
+      <c r="L7" s="27"/>
+      <c r="M7" s="26"/>
+      <c r="N7" s="26"/>
+      <c r="O7" s="26">
         <v>0</v>
       </c>
-      <c r="P7" s="25" t="s">
-        <v>226</v>
-      </c>
-      <c r="Q7" s="25" t="s">
+      <c r="P7" s="26" t="s">
         <v>227</v>
       </c>
-      <c r="R7" s="25" t="s">
+      <c r="Q7" s="26" t="s">
         <v>228</v>
       </c>
-      <c r="S7" s="25"/>
-      <c r="T7" s="25"/>
-      <c r="U7" s="25"/>
-      <c r="V7" s="25"/>
-      <c r="W7" s="25"/>
-      <c r="X7" s="25"/>
-      <c r="Y7" s="25"/>
-      <c r="Z7" s="25"/>
-      <c r="AA7" s="25" t="s">
-        <v>234</v>
+      <c r="R7" s="26" t="s">
+        <v>229</v>
+      </c>
+      <c r="S7" s="26"/>
+      <c r="T7" s="26"/>
+      <c r="U7" s="26"/>
+      <c r="V7" s="26"/>
+      <c r="W7" s="26"/>
+      <c r="X7" s="26"/>
+      <c r="Y7" s="26"/>
+      <c r="Z7" s="26"/>
+      <c r="AA7" s="26" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
@@ -7241,7 +7249,7 @@
       <c r="I8" s="14"/>
       <c r="J8" s="14"/>
       <c r="K8" s="14"/>
-      <c r="L8" s="27"/>
+      <c r="L8" s="28"/>
       <c r="M8" s="14"/>
       <c r="N8" s="14"/>
       <c r="O8" s="14"/>
@@ -7273,7 +7281,7 @@
       <c r="I9" s="14"/>
       <c r="J9" s="14"/>
       <c r="K9" s="14"/>
-      <c r="L9" s="27"/>
+      <c r="L9" s="28"/>
       <c r="M9" s="14"/>
       <c r="N9" s="14"/>
       <c r="O9" s="14"/>
@@ -7305,7 +7313,7 @@
       <c r="I10" s="14"/>
       <c r="J10" s="14"/>
       <c r="K10" s="14"/>
-      <c r="L10" s="27"/>
+      <c r="L10" s="28"/>
       <c r="M10" s="14"/>
       <c r="N10" s="14"/>
       <c r="O10" s="14"/>
@@ -7337,7 +7345,7 @@
       <c r="I11" s="14"/>
       <c r="J11" s="14"/>
       <c r="K11" s="14"/>
-      <c r="L11" s="27"/>
+      <c r="L11" s="28"/>
       <c r="M11" s="14"/>
       <c r="N11" s="14"/>
       <c r="O11" s="14"/>
@@ -7369,7 +7377,7 @@
       <c r="I12" s="14"/>
       <c r="J12" s="14"/>
       <c r="K12" s="14"/>
-      <c r="L12" s="27"/>
+      <c r="L12" s="28"/>
       <c r="M12" s="14"/>
       <c r="N12" s="14"/>
       <c r="O12" s="14"/>
@@ -7401,7 +7409,7 @@
       <c r="I13" s="14"/>
       <c r="J13" s="14"/>
       <c r="K13" s="14"/>
-      <c r="L13" s="27"/>
+      <c r="L13" s="28"/>
       <c r="M13" s="14"/>
       <c r="N13" s="14"/>
       <c r="O13" s="14"/>
@@ -7433,7 +7441,7 @@
       <c r="I14" s="14"/>
       <c r="J14" s="14"/>
       <c r="K14" s="14"/>
-      <c r="L14" s="27"/>
+      <c r="L14" s="28"/>
       <c r="M14" s="14"/>
       <c r="N14" s="14"/>
       <c r="O14" s="14"/>
@@ -7465,7 +7473,7 @@
       <c r="I15" s="14"/>
       <c r="J15" s="14"/>
       <c r="K15" s="14"/>
-      <c r="L15" s="27"/>
+      <c r="L15" s="28"/>
       <c r="M15" s="14"/>
       <c r="N15" s="14"/>
       <c r="O15" s="14"/>
@@ -7497,7 +7505,7 @@
       <c r="I16" s="14"/>
       <c r="J16" s="14"/>
       <c r="K16" s="14"/>
-      <c r="L16" s="27"/>
+      <c r="L16" s="28"/>
       <c r="M16" s="14"/>
       <c r="N16" s="14"/>
       <c r="O16" s="14"/>
@@ -7529,7 +7537,7 @@
       <c r="I17" s="14"/>
       <c r="J17" s="14"/>
       <c r="K17" s="14"/>
-      <c r="L17" s="27"/>
+      <c r="L17" s="28"/>
       <c r="M17" s="14"/>
       <c r="N17" s="14"/>
       <c r="O17" s="14"/>
@@ -7561,7 +7569,7 @@
       <c r="I18" s="14"/>
       <c r="J18" s="14"/>
       <c r="K18" s="14"/>
-      <c r="L18" s="27"/>
+      <c r="L18" s="28"/>
       <c r="M18" s="14"/>
       <c r="N18" s="14"/>
       <c r="O18" s="14"/>
@@ -7593,7 +7601,7 @@
       <c r="I19" s="14"/>
       <c r="J19" s="14"/>
       <c r="K19" s="14"/>
-      <c r="L19" s="27"/>
+      <c r="L19" s="28"/>
       <c r="M19" s="14"/>
       <c r="N19" s="14"/>
       <c r="O19" s="14"/>
@@ -7625,7 +7633,7 @@
       <c r="I20" s="14"/>
       <c r="J20" s="14"/>
       <c r="K20" s="14"/>
-      <c r="L20" s="27"/>
+      <c r="L20" s="28"/>
       <c r="M20" s="14"/>
       <c r="N20" s="14"/>
       <c r="O20" s="14"/>
@@ -7657,7 +7665,7 @@
       <c r="I21" s="14"/>
       <c r="J21" s="14"/>
       <c r="K21" s="14"/>
-      <c r="L21" s="27"/>
+      <c r="L21" s="28"/>
       <c r="M21" s="14"/>
       <c r="N21" s="14"/>
       <c r="O21" s="14"/>
@@ -7689,7 +7697,7 @@
       <c r="I22" s="14"/>
       <c r="J22" s="14"/>
       <c r="K22" s="14"/>
-      <c r="L22" s="27"/>
+      <c r="L22" s="28"/>
       <c r="M22" s="14"/>
       <c r="N22" s="14"/>
       <c r="O22" s="14"/>
@@ -7721,7 +7729,7 @@
       <c r="I23" s="14"/>
       <c r="J23" s="14"/>
       <c r="K23" s="14"/>
-      <c r="L23" s="27"/>
+      <c r="L23" s="28"/>
       <c r="M23" s="14"/>
       <c r="N23" s="14"/>
       <c r="O23" s="14"/>
@@ -7753,7 +7761,7 @@
       <c r="I24" s="14"/>
       <c r="J24" s="14"/>
       <c r="K24" s="14"/>
-      <c r="L24" s="27"/>
+      <c r="L24" s="28"/>
       <c r="M24" s="14"/>
       <c r="N24" s="14"/>
       <c r="O24" s="14"/>
@@ -7785,7 +7793,7 @@
       <c r="I25" s="14"/>
       <c r="J25" s="14"/>
       <c r="K25" s="14"/>
-      <c r="L25" s="27"/>
+      <c r="L25" s="28"/>
       <c r="M25" s="14"/>
       <c r="N25" s="14"/>
       <c r="O25" s="14"/>
@@ -7817,7 +7825,7 @@
       <c r="I26" s="14"/>
       <c r="J26" s="14"/>
       <c r="K26" s="14"/>
-      <c r="L26" s="27"/>
+      <c r="L26" s="28"/>
       <c r="M26" s="14"/>
       <c r="N26" s="14"/>
       <c r="O26" s="14"/>
@@ -7849,7 +7857,7 @@
       <c r="I27" s="14"/>
       <c r="J27" s="14"/>
       <c r="K27" s="14"/>
-      <c r="L27" s="27"/>
+      <c r="L27" s="28"/>
       <c r="M27" s="14"/>
       <c r="N27" s="14"/>
       <c r="O27" s="14"/>
@@ -7881,7 +7889,7 @@
       <c r="I28" s="14"/>
       <c r="J28" s="14"/>
       <c r="K28" s="14"/>
-      <c r="L28" s="27"/>
+      <c r="L28" s="28"/>
       <c r="M28" s="14"/>
       <c r="N28" s="14"/>
       <c r="O28" s="14"/>
@@ -7913,7 +7921,7 @@
       <c r="I29" s="14"/>
       <c r="J29" s="14"/>
       <c r="K29" s="14"/>
-      <c r="L29" s="27"/>
+      <c r="L29" s="28"/>
       <c r="M29" s="14"/>
       <c r="N29" s="14"/>
       <c r="O29" s="14"/>
@@ -7945,7 +7953,7 @@
       <c r="I30" s="14"/>
       <c r="J30" s="14"/>
       <c r="K30" s="14"/>
-      <c r="L30" s="27"/>
+      <c r="L30" s="28"/>
       <c r="M30" s="14"/>
       <c r="N30" s="14"/>
       <c r="O30" s="14"/>
@@ -7977,7 +7985,7 @@
       <c r="I31" s="14"/>
       <c r="J31" s="14"/>
       <c r="K31" s="14"/>
-      <c r="L31" s="27"/>
+      <c r="L31" s="28"/>
       <c r="M31" s="14"/>
       <c r="N31" s="14"/>
       <c r="O31" s="14"/>
@@ -8009,7 +8017,7 @@
       <c r="I32" s="14"/>
       <c r="J32" s="14"/>
       <c r="K32" s="14"/>
-      <c r="L32" s="27"/>
+      <c r="L32" s="28"/>
       <c r="M32" s="14"/>
       <c r="N32" s="14"/>
       <c r="O32" s="14"/>
@@ -8041,7 +8049,7 @@
       <c r="I33" s="14"/>
       <c r="J33" s="14"/>
       <c r="K33" s="14"/>
-      <c r="L33" s="27"/>
+      <c r="L33" s="28"/>
       <c r="M33" s="14"/>
       <c r="N33" s="14"/>
       <c r="O33" s="14"/>
@@ -8073,7 +8081,7 @@
       <c r="I34" s="14"/>
       <c r="J34" s="14"/>
       <c r="K34" s="14"/>
-      <c r="L34" s="27"/>
+      <c r="L34" s="28"/>
       <c r="M34" s="14"/>
       <c r="N34" s="14"/>
       <c r="O34" s="14"/>
@@ -8105,7 +8113,7 @@
       <c r="I35" s="14"/>
       <c r="J35" s="14"/>
       <c r="K35" s="14"/>
-      <c r="L35" s="27"/>
+      <c r="L35" s="28"/>
       <c r="M35" s="14"/>
       <c r="N35" s="14"/>
       <c r="O35" s="14"/>
@@ -8137,7 +8145,7 @@
       <c r="I36" s="14"/>
       <c r="J36" s="14"/>
       <c r="K36" s="14"/>
-      <c r="L36" s="27"/>
+      <c r="L36" s="28"/>
       <c r="M36" s="14"/>
       <c r="N36" s="14"/>
       <c r="O36" s="14"/>
@@ -8169,7 +8177,7 @@
       <c r="I37" s="14"/>
       <c r="J37" s="14"/>
       <c r="K37" s="14"/>
-      <c r="L37" s="27"/>
+      <c r="L37" s="28"/>
       <c r="M37" s="14"/>
       <c r="N37" s="14"/>
       <c r="O37" s="14"/>
@@ -8201,7 +8209,7 @@
       <c r="I38" s="14"/>
       <c r="J38" s="14"/>
       <c r="K38" s="14"/>
-      <c r="L38" s="27"/>
+      <c r="L38" s="28"/>
       <c r="M38" s="14"/>
       <c r="N38" s="14"/>
       <c r="O38" s="14"/>
@@ -8233,7 +8241,7 @@
       <c r="I39" s="14"/>
       <c r="J39" s="14"/>
       <c r="K39" s="14"/>
-      <c r="L39" s="27"/>
+      <c r="L39" s="28"/>
       <c r="M39" s="14"/>
       <c r="N39" s="14"/>
       <c r="O39" s="14"/>
@@ -8265,7 +8273,7 @@
       <c r="I40" s="14"/>
       <c r="J40" s="14"/>
       <c r="K40" s="14"/>
-      <c r="L40" s="27"/>
+      <c r="L40" s="28"/>
       <c r="M40" s="14"/>
       <c r="N40" s="14"/>
       <c r="O40" s="14"/>
@@ -8297,7 +8305,7 @@
       <c r="I41" s="14"/>
       <c r="J41" s="14"/>
       <c r="K41" s="14"/>
-      <c r="L41" s="27"/>
+      <c r="L41" s="28"/>
       <c r="M41" s="14"/>
       <c r="N41" s="14"/>
       <c r="O41" s="14"/>
@@ -8329,7 +8337,7 @@
       <c r="I42" s="14"/>
       <c r="J42" s="14"/>
       <c r="K42" s="14"/>
-      <c r="L42" s="27"/>
+      <c r="L42" s="28"/>
       <c r="M42" s="14"/>
       <c r="N42" s="14"/>
       <c r="O42" s="14"/>
@@ -8361,7 +8369,7 @@
       <c r="I43" s="14"/>
       <c r="J43" s="14"/>
       <c r="K43" s="14"/>
-      <c r="L43" s="27"/>
+      <c r="L43" s="28"/>
       <c r="M43" s="14"/>
       <c r="N43" s="14"/>
       <c r="O43" s="14"/>
@@ -8393,7 +8401,7 @@
       <c r="I44" s="14"/>
       <c r="J44" s="14"/>
       <c r="K44" s="14"/>
-      <c r="L44" s="27"/>
+      <c r="L44" s="28"/>
       <c r="M44" s="14"/>
       <c r="N44" s="14"/>
       <c r="O44" s="14"/>
@@ -8425,7 +8433,7 @@
       <c r="I45" s="14"/>
       <c r="J45" s="14"/>
       <c r="K45" s="14"/>
-      <c r="L45" s="27"/>
+      <c r="L45" s="28"/>
       <c r="M45" s="14"/>
       <c r="N45" s="14"/>
       <c r="O45" s="14"/>
@@ -8457,7 +8465,7 @@
       <c r="I46" s="14"/>
       <c r="J46" s="14"/>
       <c r="K46" s="14"/>
-      <c r="L46" s="27"/>
+      <c r="L46" s="28"/>
       <c r="M46" s="14"/>
       <c r="N46" s="14"/>
       <c r="O46" s="14"/>
@@ -8489,7 +8497,7 @@
       <c r="I47" s="14"/>
       <c r="J47" s="14"/>
       <c r="K47" s="14"/>
-      <c r="L47" s="27"/>
+      <c r="L47" s="28"/>
       <c r="M47" s="14"/>
       <c r="N47" s="14"/>
       <c r="O47" s="14"/>
@@ -8521,7 +8529,7 @@
       <c r="I48" s="14"/>
       <c r="J48" s="14"/>
       <c r="K48" s="14"/>
-      <c r="L48" s="27"/>
+      <c r="L48" s="28"/>
       <c r="M48" s="14"/>
       <c r="N48" s="14"/>
       <c r="O48" s="14"/>
@@ -8553,7 +8561,7 @@
       <c r="I49" s="14"/>
       <c r="J49" s="14"/>
       <c r="K49" s="14"/>
-      <c r="L49" s="27"/>
+      <c r="L49" s="28"/>
       <c r="M49" s="14"/>
       <c r="N49" s="14"/>
       <c r="O49" s="14"/>
@@ -8585,7 +8593,7 @@
       <c r="I50" s="14"/>
       <c r="J50" s="14"/>
       <c r="K50" s="14"/>
-      <c r="L50" s="27"/>
+      <c r="L50" s="28"/>
       <c r="M50" s="14"/>
       <c r="N50" s="14"/>
       <c r="O50" s="14"/>
@@ -8617,7 +8625,7 @@
       <c r="I51" s="14"/>
       <c r="J51" s="14"/>
       <c r="K51" s="14"/>
-      <c r="L51" s="27"/>
+      <c r="L51" s="28"/>
       <c r="M51" s="14"/>
       <c r="N51" s="14"/>
       <c r="O51" s="14"/>
@@ -8649,7 +8657,7 @@
       <c r="I52" s="14"/>
       <c r="J52" s="14"/>
       <c r="K52" s="14"/>
-      <c r="L52" s="27"/>
+      <c r="L52" s="28"/>
       <c r="M52" s="14"/>
       <c r="N52" s="14"/>
       <c r="O52" s="14"/>
@@ -8681,7 +8689,7 @@
       <c r="I53" s="14"/>
       <c r="J53" s="14"/>
       <c r="K53" s="14"/>
-      <c r="L53" s="27"/>
+      <c r="L53" s="28"/>
       <c r="M53" s="14"/>
       <c r="N53" s="14"/>
       <c r="O53" s="14"/>
@@ -8713,7 +8721,7 @@
       <c r="I54" s="14"/>
       <c r="J54" s="14"/>
       <c r="K54" s="14"/>
-      <c r="L54" s="27"/>
+      <c r="L54" s="28"/>
       <c r="M54" s="14"/>
       <c r="N54" s="14"/>
       <c r="O54" s="14"/>
@@ -8745,7 +8753,7 @@
       <c r="I55" s="14"/>
       <c r="J55" s="14"/>
       <c r="K55" s="14"/>
-      <c r="L55" s="27"/>
+      <c r="L55" s="28"/>
       <c r="M55" s="14"/>
       <c r="N55" s="14"/>
       <c r="O55" s="14"/>
@@ -8777,7 +8785,7 @@
       <c r="I56" s="14"/>
       <c r="J56" s="14"/>
       <c r="K56" s="14"/>
-      <c r="L56" s="27"/>
+      <c r="L56" s="28"/>
       <c r="M56" s="14"/>
       <c r="N56" s="14"/>
       <c r="O56" s="14"/>
@@ -8809,7 +8817,7 @@
       <c r="I57" s="14"/>
       <c r="J57" s="14"/>
       <c r="K57" s="14"/>
-      <c r="L57" s="27"/>
+      <c r="L57" s="28"/>
       <c r="M57" s="14"/>
       <c r="N57" s="14"/>
       <c r="O57" s="14"/>
@@ -8841,7 +8849,7 @@
       <c r="I58" s="14"/>
       <c r="J58" s="14"/>
       <c r="K58" s="14"/>
-      <c r="L58" s="27"/>
+      <c r="L58" s="28"/>
       <c r="M58" s="14"/>
       <c r="N58" s="14"/>
       <c r="O58" s="14"/>
@@ -8873,7 +8881,7 @@
       <c r="I59" s="14"/>
       <c r="J59" s="14"/>
       <c r="K59" s="14"/>
-      <c r="L59" s="27"/>
+      <c r="L59" s="28"/>
       <c r="M59" s="14"/>
       <c r="N59" s="14"/>
       <c r="O59" s="14"/>
@@ -8905,7 +8913,7 @@
       <c r="I60" s="14"/>
       <c r="J60" s="14"/>
       <c r="K60" s="14"/>
-      <c r="L60" s="27"/>
+      <c r="L60" s="28"/>
       <c r="M60" s="14"/>
       <c r="N60" s="14"/>
       <c r="O60" s="14"/>
@@ -8937,7 +8945,7 @@
       <c r="I61" s="14"/>
       <c r="J61" s="14"/>
       <c r="K61" s="14"/>
-      <c r="L61" s="27"/>
+      <c r="L61" s="28"/>
       <c r="M61" s="14"/>
       <c r="N61" s="14"/>
       <c r="O61" s="14"/>
@@ -8969,7 +8977,7 @@
       <c r="I62" s="14"/>
       <c r="J62" s="14"/>
       <c r="K62" s="14"/>
-      <c r="L62" s="27"/>
+      <c r="L62" s="28"/>
       <c r="M62" s="14"/>
       <c r="N62" s="14"/>
       <c r="O62" s="14"/>
@@ -9001,7 +9009,7 @@
       <c r="I63" s="14"/>
       <c r="J63" s="14"/>
       <c r="K63" s="14"/>
-      <c r="L63" s="27"/>
+      <c r="L63" s="28"/>
       <c r="M63" s="14"/>
       <c r="N63" s="14"/>
       <c r="O63" s="14"/>
@@ -9033,7 +9041,7 @@
       <c r="I64" s="14"/>
       <c r="J64" s="14"/>
       <c r="K64" s="14"/>
-      <c r="L64" s="27"/>
+      <c r="L64" s="28"/>
       <c r="M64" s="14"/>
       <c r="N64" s="14"/>
       <c r="O64" s="14"/>
@@ -9065,7 +9073,7 @@
       <c r="I65" s="14"/>
       <c r="J65" s="14"/>
       <c r="K65" s="14"/>
-      <c r="L65" s="27"/>
+      <c r="L65" s="28"/>
       <c r="M65" s="14"/>
       <c r="N65" s="14"/>
       <c r="O65" s="14"/>
@@ -9097,7 +9105,7 @@
       <c r="I66" s="14"/>
       <c r="J66" s="14"/>
       <c r="K66" s="14"/>
-      <c r="L66" s="27"/>
+      <c r="L66" s="28"/>
       <c r="M66" s="14"/>
       <c r="N66" s="14"/>
       <c r="O66" s="14"/>
@@ -9200,90 +9208,90 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="29" t="s">
-        <v>235</v>
-      </c>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
+      <c r="B1" s="30" t="s">
+        <v>236</v>
+      </c>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
     </row>
     <row r="2" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="33" t="s">
-        <v>236</v>
-      </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
+      <c r="B2" s="34" t="s">
+        <v>237</v>
+      </c>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F6" s="11" t="s">
         <v>87</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A7" s="14" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C7" s="14"/>
       <c r="D7" s="14"/>
@@ -9294,10 +9302,10 @@
     </row>
     <row r="8" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C8" s="14"/>
       <c r="D8" s="14"/>
@@ -9308,10 +9316,10 @@
     </row>
     <row r="9" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A9" s="14" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C9" s="14"/>
       <c r="D9" s="14"/>
@@ -9322,10 +9330,10 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C10" s="14"/>
       <c r="D10" s="14"/>
@@ -9336,10 +9344,10 @@
     </row>
     <row r="11" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C11" s="14"/>
       <c r="D11" s="14"/>
@@ -9350,10 +9358,10 @@
     </row>
     <row r="12" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A12" s="14" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C12" s="14"/>
       <c r="D12" s="14"/>
@@ -9364,10 +9372,10 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="14" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C13" s="14"/>
       <c r="D13" s="14"/>
@@ -9378,10 +9386,10 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C14" s="14"/>
       <c r="D14" s="14"/>
@@ -9940,50 +9948,50 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="29" t="s">
         <v>99</v>
       </c>
-      <c r="C1" s="28" t="s">
-        <v>265</v>
-      </c>
-      <c r="D1" s="28" t="s">
+      <c r="C1" s="29" t="s">
         <v>266</v>
       </c>
-      <c r="E1" s="28" t="s">
-        <v>192</v>
-      </c>
-      <c r="F1" s="28" t="s">
+      <c r="D1" s="29" t="s">
         <v>267</v>
       </c>
-      <c r="G1" s="28" t="s">
-        <v>197</v>
-      </c>
-      <c r="H1" s="28" t="s">
+      <c r="E1" s="29" t="s">
+        <v>193</v>
+      </c>
+      <c r="F1" s="29" t="s">
+        <v>268</v>
+      </c>
+      <c r="G1" s="29" t="s">
         <v>198</v>
       </c>
-      <c r="I1" s="28" t="s">
-        <v>268</v>
-      </c>
-      <c r="J1" s="28" t="s">
+      <c r="H1" s="29" t="s">
+        <v>199</v>
+      </c>
+      <c r="I1" s="29" t="s">
         <v>269</v>
       </c>
-      <c r="K1" s="28" t="s">
+      <c r="J1" s="29" t="s">
         <v>270</v>
       </c>
-      <c r="L1" s="28" t="s">
+      <c r="K1" s="29" t="s">
         <v>271</v>
       </c>
-      <c r="M1" s="28" t="s">
+      <c r="L1" s="29" t="s">
         <v>272</v>
       </c>
-      <c r="N1" s="28" t="s">
+      <c r="M1" s="29" t="s">
         <v>273</v>
       </c>
-      <c r="O1" s="28" t="s">
+      <c r="N1" s="29" t="s">
         <v>274</v>
+      </c>
+      <c r="O1" s="29" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
@@ -9997,22 +10005,22 @@
         <v>121</v>
       </c>
       <c r="D2" t="s">
+        <v>219</v>
+      </c>
+      <c r="E2" t="s">
+        <v>220</v>
+      </c>
+      <c r="F2" t="s">
         <v>218</v>
       </c>
-      <c r="E2" t="s">
-        <v>219</v>
-      </c>
-      <c r="F2" t="s">
-        <v>217</v>
-      </c>
       <c r="G2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="H2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="J2" t="s">
         <v>87</v>
@@ -10024,13 +10032,13 @@
         <v>90</v>
       </c>
       <c r="M2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="N2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="O2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
@@ -10038,46 +10046,46 @@
         <v>169</v>
       </c>
       <c r="B3" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C3" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D3" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="G3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="I3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="J3" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="K3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="L3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="M3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="N3" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="O3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
@@ -10085,75 +10093,75 @@
         <v>135</v>
       </c>
       <c r="B4" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C4" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D4" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E4" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F4" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="G4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="I4" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="K4" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="M4" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="N4" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="O4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B5" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C5" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D5" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E5" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="F5" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="G5" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="I5" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="K5" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="M5" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="N5" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="O5" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
@@ -10164,150 +10172,150 @@
         <v>115</v>
       </c>
       <c r="D6" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="F6" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="K6" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="M6" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="N6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="O6" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D7" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F7" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="M7" t="s">
         <v>86</v>
       </c>
       <c r="N7" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="O7" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D8" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="M8" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="N8" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="O8" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D9" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="M9" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="N9" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="O9" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D10" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="M10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="N10" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D11" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="M11" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="N11" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="D12" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="M12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="N12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M13" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="N13" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M14" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="N14" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M15" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="N15" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M16" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="N16" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Requirements template: five new investigation functions (BR-007)
Legal, Procurement, Finance, Cybersecurity and ARC Chairman under Report
Category Other. Access follows the Investigation Group, so each needs a
group, a routing entry and licensed members: the new 'BR-007 Impact'
sheet lists that and the decisions ERC needs to make, and the groups
are pre-filled on 'Groups & Contacts'. The impact sheet builder is now
shared by BR-006 and BR-007.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/WB-Requirements-and-SLA-Template-v1.3.xlsx
+++ b/docs/WB-Requirements-and-SLA-Template-v1.3.xlsx
@@ -12,9 +12,10 @@
     <sheet name="Request Form Fields" sheetId="3" r:id="rId3"/>
     <sheet name="Other Requirements" sheetId="4" r:id="rId4"/>
     <sheet name="BR-006 Impact" sheetId="5" r:id="rId5"/>
-    <sheet name="SLA" sheetId="6" r:id="rId6"/>
-    <sheet name="Groups &amp; Contacts" sheetId="7" r:id="rId7"/>
-    <sheet name="Lists" sheetId="8" state="hidden" r:id="rId8"/>
+    <sheet name="BR-007 Impact" sheetId="6" r:id="rId6"/>
+    <sheet name="SLA" sheetId="7" r:id="rId7"/>
+    <sheet name="Groups &amp; Contacts" sheetId="8" r:id="rId8"/>
+    <sheet name="Lists" sheetId="9" state="hidden" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="Area">Lists!$A$2:$A$11</definedName>
@@ -22,7 +23,7 @@
     <definedName name="Channel">Lists!$I$2:$I$5</definedName>
     <definedName name="FieldType">Lists!$M$2:$M$16</definedName>
     <definedName name="FilledBy">Lists!$L$2:$L$3</definedName>
-    <definedName name="GroupNames">Lists!$O$2:$O$9</definedName>
+    <definedName name="GroupNames">Lists!$O$2:$O$14</definedName>
     <definedName name="JiraField">Lists!$N$2:$N$16</definedName>
     <definedName name="Priority">Lists!$B$2:$B$5</definedName>
     <definedName name="ReportCategory">Lists!$D$2:$D$12</definedName>
@@ -345,7 +346,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="397">
   <si>
     <t>Whistleblowing Reporting Portal - Requirements Template</t>
   </si>
@@ -405,6 +406,12 @@
   </si>
   <si>
     <t>What the escalation branch (BR-006) changes in today's setup, and the decisions needed - answer in the yellow 'ERC answer' cells.</t>
+  </si>
+  <si>
+    <t>BR-007 Impact</t>
+  </si>
+  <si>
+    <t>The same for the five new investigation functions (BR-007).</t>
   </si>
   <si>
     <t>SLA</t>
@@ -800,6 +807,24 @@
     <t>11 impacted areas and the decisions ERC needs to make are listed on the 'BR-006 Impact' sheet.</t>
   </si>
   <si>
+    <t>Five more investigation functions under Report Category "Other"</t>
+  </si>
+  <si>
+    <t>When the Report Category is "Other", the Compliance Manager chooses the Investigating Function. Add these functions, each with its own investigation group:
+1. Legal
+2. Procurement
+3. Finance
+4. Cybersecurity
+5. ARC Chairman
+This affects the investigation group, the assignee and the user groups. Impact on current areas: see the 'BR-007 Impact' sheet.</t>
+  </si>
+  <si>
+    <t>Choosing each new function on a test report routes it to that function's group only: its members get the assignment email, can be assigned and can see the report; no other investigation group can.</t>
+  </si>
+  <si>
+    <t>Groups added to the 'Groups &amp; Contacts' sheet for ERC to fill in the members. Decisions needed are on the 'BR-007 Impact' sheet.</t>
+  </si>
+  <si>
     <t>BR-006 - Impact of the escalation branch</t>
   </si>
   <si>
@@ -938,6 +963,120 @@
     <t>No change: the questions apply to new reports only.</t>
   </si>
   <si>
+    <t>BR-007 - Impact of the five new investigation functions</t>
+  </si>
+  <si>
+    <t>What changes when Legal, Procurement, Finance, Cybersecurity and ARC Chairman can investigate</t>
+  </si>
+  <si>
+    <t>Access to a report follows its Investigation Group, so each new function needs a group, a routing entry and licensed members - nothing else in the workflow changes.</t>
+  </si>
+  <si>
+    <t>Investigating Function (form question)</t>
+  </si>
+  <si>
+    <t>Shown when the Report Category is Other. Options: Internal Audit, Human Resources, Health and Safety representative, Information Security, GRC-Compliance Manager.</t>
+  </si>
+  <si>
+    <t>Add the five options to the Compliance Approval form and to the Investigating Function field: Legal, Procurement, Finance, Cybersecurity, ARC Chairman.</t>
+  </si>
+  <si>
+    <t>Confirm the Arabic labels for the five options.</t>
+  </si>
+  <si>
+    <t>Investigation Group</t>
+  </si>
+  <si>
+    <t>Set automatically from the Investigating Function when the Compliance Manager submits the form; one group per function.</t>
+  </si>
+  <si>
+    <t>Five new Jira groups, and the five function-to-group pairs added to the routing rule.</t>
+  </si>
+  <si>
+    <t>Group names. Jira groups are shared across ERC's whole Atlassian organisation: a generic name such as "Finance" may already exist with all finance staff in it, and every one of them would see these reports. Dedicated names (e.g. "WB-Finance") are safer.</t>
+  </si>
+  <si>
+    <t>Group members</t>
+  </si>
+  <si>
+    <t>One row per new group added to the 'Groups &amp; Contacts' sheet.</t>
+  </si>
+  <si>
+    <t>Members and emails for each group.</t>
+  </si>
+  <si>
+    <t>Assignee</t>
+  </si>
+  <si>
+    <t>Members of GRC-Compliance and of the report's Investigation Group can be assigned.</t>
+  </si>
+  <si>
+    <t>No permission change: members of a new group can be assigned as soon as a report is routed to it.</t>
+  </si>
+  <si>
+    <t>Who in each group should be assigned first, if anyone (default assignee)?</t>
+  </si>
+  <si>
+    <t>A report is visible to GRC-Compliance and to its Investigation Group only.</t>
+  </si>
+  <si>
+    <t>No change to the security level: each new group sees only the reports routed to it.</t>
+  </si>
+  <si>
+    <t>Licences and sign-in</t>
+  </si>
+  <si>
+    <t>Every investigator needs a Jira Service Management agent licence and must be assigned to the "Jira - SSO" enterprise app in Entra ID.</t>
+  </si>
+  <si>
+    <t>Members of the five groups need agent licences and the SSO assignment before go-live.</t>
+  </si>
+  <si>
+    <t>Are enough agent licences available for the new members?</t>
+  </si>
+  <si>
+    <t>ARC Chairman</t>
+  </si>
+  <si>
+    <t>A single person, possibly outside ERC's staff directory. As an investigation function they would need a Jira account, a licence, and would see the full report in Jira.</t>
+  </si>
+  <si>
+    <t>Should the ARC Chairman work in Jira, or receive these cases another way (e.g. through Internal Audit)?</t>
+  </si>
+  <si>
+    <t>Cybersecurity and Information Security</t>
+  </si>
+  <si>
+    <t>Information Security investigates information security and data protection reports.</t>
+  </si>
+  <si>
+    <t>Cybersecurity is added as a separate function. Under BR-006, a report about the Cybersecurity department goes to Internal Audit, so Cybersecurity never investigates a report about itself.</t>
+  </si>
+  <si>
+    <t>Is Cybersecurity a different team from Information Security, or the same group?</t>
+  </si>
+  <si>
+    <t>The assignment email goes to the report's Investigation Group.</t>
+  </si>
+  <si>
+    <t>Works for the new groups once they are in the routing rule.</t>
+  </si>
+  <si>
+    <t>Investigation decision: 2 working days, for every investigation group.</t>
+  </si>
+  <si>
+    <t>Applies to the new groups automatically.</t>
+  </si>
+  <si>
+    <t>Documentation and reporting</t>
+  </si>
+  <si>
+    <t>The user guide lists the groups and the category-to-function table. Power BI breaks reports down by group.</t>
+  </si>
+  <si>
+    <t>Update the guide's tables; the new functions appear in reporting once used.</t>
+  </si>
+  <si>
     <t>Service Levels (SLA) and Escalation</t>
   </si>
   <si>
@@ -1176,6 +1315,33 @@
   </si>
   <si>
     <t>Oversight: sees all reports</t>
+  </si>
+  <si>
+    <t>Legal</t>
+  </si>
+  <si>
+    <t>Investigates reports routed to Legal (Report Category Other) - new, BR-007</t>
+  </si>
+  <si>
+    <t>Procurement</t>
+  </si>
+  <si>
+    <t>Investigates reports routed to Procurement (Report Category Other) - new, BR-007</t>
+  </si>
+  <si>
+    <t>Finance</t>
+  </si>
+  <si>
+    <t>Investigates reports routed to Finance (Report Category Other) - new, BR-007</t>
+  </si>
+  <si>
+    <t>Cybersecurity</t>
+  </si>
+  <si>
+    <t>Investigates reports routed to Cybersecurity (Report Category Other) - new, BR-007</t>
+  </si>
+  <si>
+    <t>Investigates reports routed to ARC Chairman (Report Category Other) - new, BR-007</t>
   </si>
   <si>
     <t>ReqStatus</t>
@@ -1860,6 +2026,38 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="438150" cy="390525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2148,7 +2346,7 @@
   <sheetPr>
     <tabColor rgb="FF024638"/>
   </sheetPr>
-  <dimension ref="B1:C35"/>
+  <dimension ref="B1:C36"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -2242,7 +2440,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="2:3" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>20</v>
       </c>
@@ -2250,7 +2448,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:3" ht="26.4" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
         <v>22</v>
       </c>
@@ -2258,16 +2456,16 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B18" s="1" t="s">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B17" s="5" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B19" s="5" t="s">
+      <c r="C17" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="6" t="s">
+    </row>
+    <row r="19" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B19" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2299,89 +2497,97 @@
       <c r="B23" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C23" s="7"/>
+      <c r="C23" s="6" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B24" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C24" s="7"/>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B25" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C25" s="7"/>
     </row>
-    <row r="27" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B27" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B28" s="5" t="s">
+    <row r="26" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B26" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C28" s="8">
+      <c r="C26" s="7"/>
+    </row>
+    <row r="28" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B28" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B29" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C29" s="8">
         <f>COUNTA('Service Catalog'!C7:C66)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B29" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="C29" s="8">
+    <row r="30" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B30" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C30" s="8">
         <f>COUNTA('Request Form Fields'!D7:D66)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B30" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C30" s="8">
-        <f>COUNTA('Other Requirements'!C7:C66)</f>
-        <v>5</v>
-      </c>
-    </row>
     <row r="31" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B31" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C31" s="8">
+        <f>COUNTA('Other Requirements'!C7:C66)</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B32" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C32" s="8">
         <f>COUNTIF('Other Requirements'!K7:K66,"Approved")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B32" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="C32" s="8">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B33" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C33" s="8">
         <f>COUNTA(SLA!B7:B66)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B33" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C33" s="8">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B34" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C34" s="8">
         <f>COUNTA('Groups &amp; Contacts'!C7:C66)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B35" s="32" t="s">
-        <v>43</v>
-      </c>
-      <c r="C35" s="33"/>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B36" s="32" t="s">
+        <v>45</v>
+      </c>
+      <c r="C36" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
     <mergeCell ref="B2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2429,7 +2635,7 @@
     </row>
     <row r="2" spans="1:14" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="34" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C2" s="31"/>
       <c r="D2" s="31"/>
@@ -2446,86 +2652,86 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="M5" s="10" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J6" s="11" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="L6" s="12">
         <f t="shared" ref="L6:L37" si="0">IF(C6="","",SUMPRODUCT((TRIM(F6:H6)&lt;&gt;"")*(TRIM(F6:H6)&lt;&gt;"None")*(TRIM(F6:H6)&lt;&gt;"-")))</f>
@@ -2536,7 +2742,7 @@
         <v>1</v>
       </c>
       <c r="N6" s="11" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
@@ -4094,7 +4300,7 @@
     </row>
     <row r="2" spans="1:12" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="34" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C2" s="31"/>
       <c r="D2" s="31"/>
@@ -4109,84 +4315,84 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C6" s="11">
         <v>1</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="J6" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="K6" s="11" t="str">
         <f t="shared" ref="K6:K37" si="0">IF(F6="","",IFERROR(INDEX(JiraField,MATCH(F6,FieldType,0)),"Ejada to review"))</f>
         <v>Select List (single choice)</v>
       </c>
       <c r="L6" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
@@ -5455,7 +5661,7 @@
     </row>
     <row r="2" spans="1:12" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="34" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C2" s="31"/>
       <c r="D2" s="31"/>
@@ -5470,83 +5676,83 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="J6" s="16" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="L6" s="11" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="52.8" x14ac:dyDescent="0.3">
@@ -5555,27 +5761,27 @@
         <v>BR-002</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E7" s="14"/>
       <c r="F7" s="14"/>
       <c r="G7" s="14"/>
       <c r="H7" s="14"/>
       <c r="I7" s="14" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="J7" s="17"/>
       <c r="K7" s="14" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="L7" s="14" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="79.2" x14ac:dyDescent="0.3">
@@ -5584,27 +5790,27 @@
         <v>BR-003</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
       <c r="G8" s="14"/>
       <c r="H8" s="14"/>
       <c r="I8" s="14" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="J8" s="17"/>
       <c r="K8" s="14" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="L8" s="14" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="92.4" x14ac:dyDescent="0.3">
@@ -5613,27 +5819,27 @@
         <v>BR-004</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E9" s="14"/>
       <c r="F9" s="14"/>
       <c r="G9" s="14"/>
       <c r="H9" s="14"/>
       <c r="I9" s="14" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="J9" s="17"/>
       <c r="K9" s="14" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="L9" s="14" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="409.6" x14ac:dyDescent="0.3">
@@ -5642,27 +5848,27 @@
         <v>BR-005</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E10" s="14"/>
       <c r="F10" s="14"/>
       <c r="G10" s="14"/>
       <c r="H10" s="14"/>
       <c r="I10" s="14" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="J10" s="17"/>
       <c r="K10" s="14" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="L10" s="14" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="184.8" x14ac:dyDescent="0.3">
@@ -5671,45 +5877,57 @@
         <v>BR-006</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E11" s="14"/>
       <c r="F11" s="14"/>
       <c r="G11" s="14"/>
       <c r="H11" s="14"/>
       <c r="I11" s="14" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J11" s="17"/>
       <c r="K11" s="14" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="L11" s="14" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
+        <v>BR-007</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>143</v>
+      </c>
       <c r="E12" s="14"/>
       <c r="F12" s="14"/>
       <c r="G12" s="14"/>
       <c r="H12" s="14"/>
-      <c r="I12" s="14"/>
+      <c r="I12" s="14" t="s">
+        <v>144</v>
+      </c>
       <c r="J12" s="17"/>
-      <c r="K12" s="14"/>
-      <c r="L12" s="14"/>
+      <c r="K12" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="L12" s="14" t="s">
+        <v>145</v>
+      </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="13" t="str">
@@ -6672,7 +6890,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="30" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="C1" s="31"/>
       <c r="D1" s="31"/>
@@ -6681,7 +6899,7 @@
     </row>
     <row r="2" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="34" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="C2" s="31"/>
       <c r="D2" s="31"/>
@@ -6690,27 +6908,27 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="18" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
@@ -6718,16 +6936,16 @@
         <v>1</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="F6" s="14"/>
     </row>
@@ -6736,16 +6954,16 @@
         <v>2</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="F7" s="14"/>
     </row>
@@ -6754,16 +6972,16 @@
         <v>3</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F8" s="23"/>
     </row>
@@ -6772,16 +6990,16 @@
         <v>4</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="F9" s="14"/>
     </row>
@@ -6790,16 +7008,16 @@
         <v>5</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F10" s="23"/>
     </row>
@@ -6808,16 +7026,16 @@
         <v>6</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="F11" s="14"/>
     </row>
@@ -6826,16 +7044,16 @@
         <v>7</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="F12" s="14"/>
     </row>
@@ -6844,16 +7062,16 @@
         <v>8</v>
       </c>
       <c r="B13" s="22" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="F13" s="14"/>
     </row>
@@ -6862,19 +7080,19 @@
         <v>9</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="F14" s="24" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
@@ -6882,16 +7100,16 @@
         <v>10</v>
       </c>
       <c r="B15" s="22" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="C15" s="21" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F15" s="23"/>
     </row>
@@ -6900,16 +7118,16 @@
         <v>11</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F16" s="23"/>
     </row>
@@ -6924,6 +7142,273 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FF024638"/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="42" customWidth="1"/>
+    <col min="4" max="4" width="52" customWidth="1"/>
+    <col min="5" max="5" width="46" customWidth="1"/>
+    <col min="6" max="6" width="40" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="30" t="s">
+        <v>192</v>
+      </c>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+    </row>
+    <row r="2" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="34" t="s">
+        <v>193</v>
+      </c>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="E5" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="F5" s="18" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="19">
+        <v>1</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>195</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>196</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>197</v>
+      </c>
+      <c r="E6" s="19" t="s">
+        <v>198</v>
+      </c>
+      <c r="F6" s="14"/>
+    </row>
+    <row r="7" spans="1:6" ht="66" x14ac:dyDescent="0.3">
+      <c r="A7" s="21">
+        <v>2</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>199</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>200</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>201</v>
+      </c>
+      <c r="E7" s="21" t="s">
+        <v>202</v>
+      </c>
+      <c r="F7" s="14"/>
+    </row>
+    <row r="8" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A8" s="19">
+        <v>3</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>203</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>204</v>
+      </c>
+      <c r="E8" s="19" t="s">
+        <v>205</v>
+      </c>
+      <c r="F8" s="14"/>
+    </row>
+    <row r="9" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="21">
+        <v>4</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>206</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>207</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>208</v>
+      </c>
+      <c r="E9" s="21" t="s">
+        <v>209</v>
+      </c>
+      <c r="F9" s="14"/>
+    </row>
+    <row r="10" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A10" s="19">
+        <v>5</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>165</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>210</v>
+      </c>
+      <c r="D10" s="19" t="s">
+        <v>211</v>
+      </c>
+      <c r="E10" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="F10" s="23"/>
+    </row>
+    <row r="11" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="21">
+        <v>6</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>212</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>213</v>
+      </c>
+      <c r="D11" s="21" t="s">
+        <v>214</v>
+      </c>
+      <c r="E11" s="21" t="s">
+        <v>215</v>
+      </c>
+      <c r="F11" s="14"/>
+    </row>
+    <row r="12" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="19">
+        <v>7</v>
+      </c>
+      <c r="B12" s="20" t="s">
+        <v>216</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="D12" s="19" t="s">
+        <v>217</v>
+      </c>
+      <c r="E12" s="19" t="s">
+        <v>218</v>
+      </c>
+      <c r="F12" s="14"/>
+    </row>
+    <row r="13" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="21">
+        <v>8</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>219</v>
+      </c>
+      <c r="C13" s="21" t="s">
+        <v>220</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>221</v>
+      </c>
+      <c r="E13" s="21" t="s">
+        <v>222</v>
+      </c>
+      <c r="F13" s="14"/>
+    </row>
+    <row r="14" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A14" s="19">
+        <v>9</v>
+      </c>
+      <c r="B14" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>223</v>
+      </c>
+      <c r="D14" s="19" t="s">
+        <v>224</v>
+      </c>
+      <c r="E14" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="F14" s="23"/>
+    </row>
+    <row r="15" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A15" s="21">
+        <v>10</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>171</v>
+      </c>
+      <c r="C15" s="21" t="s">
+        <v>225</v>
+      </c>
+      <c r="D15" s="21" t="s">
+        <v>226</v>
+      </c>
+      <c r="E15" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="F15" s="23"/>
+    </row>
+    <row r="16" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="19">
+        <v>11</v>
+      </c>
+      <c r="B16" s="20" t="s">
+        <v>227</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>228</v>
+      </c>
+      <c r="D16" s="19" t="s">
+        <v>229</v>
+      </c>
+      <c r="E16" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="F16" s="23"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF024638"/>
@@ -6959,7 +7444,7 @@
   <sheetData>
     <row r="1" spans="1:27" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="30" t="s">
-        <v>186</v>
+        <v>230</v>
       </c>
       <c r="C1" s="31"/>
       <c r="D1" s="31"/>
@@ -6989,7 +7474,7 @@
     </row>
     <row r="2" spans="1:27" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="34" t="s">
-        <v>187</v>
+        <v>231</v>
       </c>
       <c r="C2" s="31"/>
       <c r="D2" s="31"/>
@@ -7019,144 +7504,144 @@
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>188</v>
+        <v>232</v>
       </c>
     </row>
     <row r="5" spans="1:27" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>189</v>
+        <v>233</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>190</v>
+        <v>234</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>191</v>
+        <v>235</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>192</v>
+        <v>236</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>193</v>
+        <v>237</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>194</v>
+        <v>238</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>195</v>
+        <v>239</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>196</v>
+        <v>240</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>197</v>
+        <v>241</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>198</v>
+        <v>242</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>199</v>
+        <v>243</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>200</v>
+        <v>244</v>
       </c>
       <c r="M5" s="10" t="s">
-        <v>201</v>
+        <v>245</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>202</v>
+        <v>246</v>
       </c>
       <c r="O5" s="10" t="s">
-        <v>203</v>
+        <v>247</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="Q5" s="10" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
       <c r="R5" s="10" t="s">
-        <v>206</v>
+        <v>250</v>
       </c>
       <c r="S5" s="10" t="s">
-        <v>207</v>
+        <v>251</v>
       </c>
       <c r="T5" s="10" t="s">
-        <v>208</v>
+        <v>252</v>
       </c>
       <c r="U5" s="10" t="s">
-        <v>209</v>
+        <v>253</v>
       </c>
       <c r="V5" s="10" t="s">
-        <v>210</v>
+        <v>254</v>
       </c>
       <c r="W5" s="10" t="s">
-        <v>211</v>
+        <v>255</v>
       </c>
       <c r="X5" s="10" t="s">
-        <v>212</v>
+        <v>256</v>
       </c>
       <c r="Y5" s="10" t="s">
-        <v>213</v>
+        <v>257</v>
       </c>
       <c r="Z5" s="10" t="s">
-        <v>214</v>
+        <v>258</v>
       </c>
       <c r="AA5" s="10" t="s">
-        <v>215</v>
+        <v>259</v>
       </c>
     </row>
     <row r="6" spans="1:27" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>217</v>
+        <v>261</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>218</v>
+        <v>262</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>219</v>
+        <v>263</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>220</v>
+        <v>264</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>221</v>
+        <v>265</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>222</v>
+        <v>266</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>223</v>
+        <v>267</v>
       </c>
       <c r="I6" s="11">
         <v>2</v>
       </c>
       <c r="J6" s="11" t="s">
-        <v>224</v>
+        <v>268</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>225</v>
+        <v>269</v>
       </c>
       <c r="L6" s="25">
         <v>0.75</v>
       </c>
       <c r="M6" s="11" t="s">
-        <v>226</v>
+        <v>270</v>
       </c>
       <c r="N6" s="11"/>
       <c r="O6" s="11">
         <v>0</v>
       </c>
       <c r="P6" s="11" t="s">
-        <v>227</v>
+        <v>271</v>
       </c>
       <c r="Q6" s="11" t="s">
-        <v>228</v>
+        <v>272</v>
       </c>
       <c r="R6" s="11" t="s">
-        <v>229</v>
+        <v>273</v>
       </c>
       <c r="S6" s="11">
         <v>1</v>
@@ -7169,7 +7654,7 @@
       <c r="Y6" s="11"/>
       <c r="Z6" s="11"/>
       <c r="AA6" s="11" t="s">
-        <v>230</v>
+        <v>274</v>
       </c>
     </row>
     <row r="7" spans="1:27" ht="26.4" x14ac:dyDescent="0.3">
@@ -7178,34 +7663,34 @@
         <v>SLA-02</v>
       </c>
       <c r="B7" s="26" t="s">
-        <v>231</v>
+        <v>275</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>232</v>
+        <v>276</v>
       </c>
       <c r="D7" s="26" t="s">
-        <v>219</v>
+        <v>263</v>
       </c>
       <c r="E7" s="26" t="s">
-        <v>220</v>
+        <v>264</v>
       </c>
       <c r="F7" s="26" t="s">
-        <v>233</v>
+        <v>277</v>
       </c>
       <c r="G7" s="26" t="s">
-        <v>234</v>
+        <v>278</v>
       </c>
       <c r="H7" s="26" t="s">
-        <v>223</v>
+        <v>267</v>
       </c>
       <c r="I7" s="26">
         <v>2</v>
       </c>
       <c r="J7" s="26" t="s">
-        <v>224</v>
+        <v>268</v>
       </c>
       <c r="K7" s="26" t="s">
-        <v>225</v>
+        <v>269</v>
       </c>
       <c r="L7" s="27"/>
       <c r="M7" s="26"/>
@@ -7214,13 +7699,13 @@
         <v>0</v>
       </c>
       <c r="P7" s="26" t="s">
-        <v>227</v>
+        <v>271</v>
       </c>
       <c r="Q7" s="26" t="s">
-        <v>228</v>
+        <v>272</v>
       </c>
       <c r="R7" s="26" t="s">
-        <v>229</v>
+        <v>273</v>
       </c>
       <c r="S7" s="26"/>
       <c r="T7" s="26"/>
@@ -7231,7 +7716,7 @@
       <c r="Y7" s="26"/>
       <c r="Z7" s="26"/>
       <c r="AA7" s="26" t="s">
-        <v>235</v>
+        <v>279</v>
       </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
@@ -9190,7 +9675,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF36B78E"/>
@@ -9209,7 +9694,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="30" t="s">
-        <v>236</v>
+        <v>280</v>
       </c>
       <c r="C1" s="31"/>
       <c r="D1" s="31"/>
@@ -9220,7 +9705,7 @@
     </row>
     <row r="2" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="34" t="s">
-        <v>237</v>
+        <v>281</v>
       </c>
       <c r="C2" s="31"/>
       <c r="D2" s="31"/>
@@ -9231,67 +9716,67 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>238</v>
+        <v>282</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>239</v>
+        <v>283</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>240</v>
+        <v>284</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>241</v>
+        <v>285</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>242</v>
+        <v>286</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>243</v>
+        <v>287</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>244</v>
+        <v>288</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>245</v>
+        <v>289</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>215</v>
+        <v>259</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>226</v>
+        <v>270</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>246</v>
+        <v>290</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>247</v>
+        <v>291</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>248</v>
+        <v>292</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>249</v>
+        <v>293</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>250</v>
+        <v>294</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>251</v>
+        <v>295</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A7" s="14" t="s">
-        <v>226</v>
+        <v>270</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>252</v>
+        <v>296</v>
       </c>
       <c r="C7" s="14"/>
       <c r="D7" s="14"/>
@@ -9302,10 +9787,10 @@
     </row>
     <row r="8" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
-        <v>253</v>
+        <v>297</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>254</v>
+        <v>298</v>
       </c>
       <c r="C8" s="14"/>
       <c r="D8" s="14"/>
@@ -9316,10 +9801,10 @@
     </row>
     <row r="9" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A9" s="14" t="s">
-        <v>255</v>
+        <v>299</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>256</v>
+        <v>300</v>
       </c>
       <c r="C9" s="14"/>
       <c r="D9" s="14"/>
@@ -9330,10 +9815,10 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
-        <v>257</v>
+        <v>301</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>258</v>
+        <v>302</v>
       </c>
       <c r="C10" s="14"/>
       <c r="D10" s="14"/>
@@ -9344,10 +9829,10 @@
     </row>
     <row r="11" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
-        <v>259</v>
+        <v>303</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>260</v>
+        <v>304</v>
       </c>
       <c r="C11" s="14"/>
       <c r="D11" s="14"/>
@@ -9358,10 +9843,10 @@
     </row>
     <row r="12" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A12" s="14" t="s">
-        <v>261</v>
+        <v>305</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>262</v>
+        <v>306</v>
       </c>
       <c r="C12" s="14"/>
       <c r="D12" s="14"/>
@@ -9372,10 +9857,10 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="14" t="s">
-        <v>227</v>
+        <v>271</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>263</v>
+        <v>307</v>
       </c>
       <c r="C13" s="14"/>
       <c r="D13" s="14"/>
@@ -9386,10 +9871,10 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="14" t="s">
-        <v>264</v>
+        <v>308</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>265</v>
+        <v>309</v>
       </c>
       <c r="C14" s="14"/>
       <c r="D14" s="14"/>
@@ -9398,9 +9883,13 @@
       <c r="G14" s="14"/>
       <c r="H14" s="14"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="14"/>
-      <c r="B15" s="14"/>
+    <row r="15" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A15" s="14" t="s">
+        <v>310</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>311</v>
+      </c>
       <c r="C15" s="14"/>
       <c r="D15" s="14"/>
       <c r="E15" s="14"/>
@@ -9408,9 +9897,13 @@
       <c r="G15" s="14"/>
       <c r="H15" s="14"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="14"/>
-      <c r="B16" s="14"/>
+    <row r="16" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A16" s="14" t="s">
+        <v>312</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>313</v>
+      </c>
       <c r="C16" s="14"/>
       <c r="D16" s="14"/>
       <c r="E16" s="14"/>
@@ -9418,9 +9911,13 @@
       <c r="G16" s="14"/>
       <c r="H16" s="14"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="14"/>
-      <c r="B17" s="14"/>
+    <row r="17" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A17" s="14" t="s">
+        <v>314</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>315</v>
+      </c>
       <c r="C17" s="14"/>
       <c r="D17" s="14"/>
       <c r="E17" s="14"/>
@@ -9428,9 +9925,13 @@
       <c r="G17" s="14"/>
       <c r="H17" s="14"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="14"/>
-      <c r="B18" s="14"/>
+    <row r="18" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A18" s="14" t="s">
+        <v>316</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>317</v>
+      </c>
       <c r="C18" s="14"/>
       <c r="D18" s="14"/>
       <c r="E18" s="14"/>
@@ -9438,9 +9939,13 @@
       <c r="G18" s="14"/>
       <c r="H18" s="14"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="14"/>
-      <c r="B19" s="14"/>
+    <row r="19" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A19" s="14" t="s">
+        <v>216</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>318</v>
+      </c>
       <c r="C19" s="14"/>
       <c r="D19" s="14"/>
       <c r="E19" s="14"/>
@@ -9942,380 +10447,395 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="29" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B1" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C1" s="29" t="s">
-        <v>266</v>
+        <v>319</v>
       </c>
       <c r="D1" s="29" t="s">
-        <v>267</v>
+        <v>320</v>
       </c>
       <c r="E1" s="29" t="s">
-        <v>193</v>
+        <v>237</v>
       </c>
       <c r="F1" s="29" t="s">
-        <v>268</v>
+        <v>321</v>
       </c>
       <c r="G1" s="29" t="s">
-        <v>198</v>
+        <v>242</v>
       </c>
       <c r="H1" s="29" t="s">
-        <v>199</v>
+        <v>243</v>
       </c>
       <c r="I1" s="29" t="s">
-        <v>269</v>
+        <v>322</v>
       </c>
       <c r="J1" s="29" t="s">
-        <v>270</v>
+        <v>323</v>
       </c>
       <c r="K1" s="29" t="s">
-        <v>271</v>
+        <v>324</v>
       </c>
       <c r="L1" s="29" t="s">
-        <v>272</v>
+        <v>325</v>
       </c>
       <c r="M1" s="29" t="s">
-        <v>273</v>
+        <v>326</v>
       </c>
       <c r="N1" s="29" t="s">
-        <v>274</v>
+        <v>327</v>
       </c>
       <c r="O1" s="29" t="s">
-        <v>275</v>
+        <v>328</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D2" t="s">
-        <v>219</v>
+        <v>263</v>
       </c>
       <c r="E2" t="s">
-        <v>220</v>
+        <v>264</v>
       </c>
       <c r="F2" t="s">
-        <v>218</v>
+        <v>262</v>
       </c>
       <c r="G2" t="s">
-        <v>276</v>
+        <v>329</v>
       </c>
       <c r="H2" t="s">
-        <v>225</v>
+        <v>269</v>
       </c>
       <c r="I2" t="s">
-        <v>229</v>
+        <v>273</v>
       </c>
       <c r="J2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="K2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="L2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="M2" t="s">
-        <v>277</v>
+        <v>330</v>
       </c>
       <c r="N2" t="s">
-        <v>278</v>
+        <v>331</v>
       </c>
       <c r="O2" t="s">
-        <v>226</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="B3" t="s">
-        <v>279</v>
+        <v>332</v>
       </c>
       <c r="C3" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D3" t="s">
-        <v>281</v>
+        <v>334</v>
       </c>
       <c r="E3" t="s">
-        <v>282</v>
+        <v>335</v>
       </c>
       <c r="F3" t="s">
-        <v>232</v>
+        <v>276</v>
       </c>
       <c r="G3" t="s">
-        <v>224</v>
+        <v>268</v>
       </c>
       <c r="H3" t="s">
-        <v>283</v>
+        <v>336</v>
       </c>
       <c r="I3" t="s">
-        <v>284</v>
+        <v>337</v>
       </c>
       <c r="J3" t="s">
-        <v>250</v>
+        <v>294</v>
       </c>
       <c r="K3" t="s">
-        <v>285</v>
+        <v>338</v>
       </c>
       <c r="L3" t="s">
-        <v>286</v>
+        <v>339</v>
       </c>
       <c r="M3" t="s">
-        <v>287</v>
+        <v>340</v>
       </c>
       <c r="N3" t="s">
-        <v>288</v>
+        <v>341</v>
       </c>
       <c r="O3" t="s">
-        <v>253</v>
+        <v>297</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B4" t="s">
-        <v>289</v>
+        <v>342</v>
       </c>
       <c r="C4" t="s">
-        <v>290</v>
+        <v>343</v>
       </c>
       <c r="D4" t="s">
-        <v>291</v>
+        <v>344</v>
       </c>
       <c r="E4" t="s">
-        <v>292</v>
+        <v>345</v>
       </c>
       <c r="F4" t="s">
-        <v>293</v>
+        <v>346</v>
       </c>
       <c r="G4" t="s">
-        <v>294</v>
+        <v>347</v>
       </c>
       <c r="I4" t="s">
-        <v>295</v>
+        <v>348</v>
       </c>
       <c r="K4" t="s">
-        <v>296</v>
+        <v>349</v>
       </c>
       <c r="M4" t="s">
-        <v>297</v>
+        <v>350</v>
       </c>
       <c r="N4" t="s">
-        <v>298</v>
+        <v>351</v>
       </c>
       <c r="O4" t="s">
-        <v>255</v>
+        <v>299</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>299</v>
+        <v>352</v>
       </c>
       <c r="B5" t="s">
-        <v>300</v>
+        <v>353</v>
       </c>
       <c r="C5" t="s">
+        <v>354</v>
+      </c>
+      <c r="D5" t="s">
+        <v>355</v>
+      </c>
+      <c r="E5" t="s">
+        <v>356</v>
+      </c>
+      <c r="F5" t="s">
+        <v>357</v>
+      </c>
+      <c r="G5" t="s">
+        <v>358</v>
+      </c>
+      <c r="I5" t="s">
+        <v>359</v>
+      </c>
+      <c r="K5" t="s">
+        <v>360</v>
+      </c>
+      <c r="M5" t="s">
+        <v>361</v>
+      </c>
+      <c r="N5" t="s">
+        <v>362</v>
+      </c>
+      <c r="O5" t="s">
         <v>301</v>
-      </c>
-      <c r="D5" t="s">
-        <v>302</v>
-      </c>
-      <c r="E5" t="s">
-        <v>303</v>
-      </c>
-      <c r="F5" t="s">
-        <v>304</v>
-      </c>
-      <c r="G5" t="s">
-        <v>305</v>
-      </c>
-      <c r="I5" t="s">
-        <v>306</v>
-      </c>
-      <c r="K5" t="s">
-        <v>307</v>
-      </c>
-      <c r="M5" t="s">
-        <v>308</v>
-      </c>
-      <c r="N5" t="s">
-        <v>309</v>
-      </c>
-      <c r="O5" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D6" t="s">
-        <v>310</v>
+        <v>363</v>
       </c>
       <c r="E6" t="s">
-        <v>311</v>
+        <v>364</v>
       </c>
       <c r="F6" t="s">
-        <v>312</v>
+        <v>365</v>
       </c>
       <c r="K6" t="s">
-        <v>313</v>
+        <v>366</v>
       </c>
       <c r="M6" t="s">
-        <v>314</v>
+        <v>367</v>
       </c>
       <c r="N6" t="s">
-        <v>315</v>
+        <v>368</v>
       </c>
       <c r="O6" t="s">
-        <v>259</v>
+        <v>303</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>316</v>
+        <v>369</v>
       </c>
       <c r="D7" t="s">
-        <v>317</v>
+        <v>370</v>
       </c>
       <c r="F7" t="s">
-        <v>318</v>
+        <v>371</v>
       </c>
       <c r="M7" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="N7" t="s">
-        <v>319</v>
+        <v>372</v>
       </c>
       <c r="O7" t="s">
-        <v>261</v>
+        <v>305</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>320</v>
+        <v>373</v>
       </c>
       <c r="D8" t="s">
-        <v>321</v>
+        <v>374</v>
       </c>
       <c r="M8" t="s">
-        <v>322</v>
+        <v>375</v>
       </c>
       <c r="N8" t="s">
-        <v>323</v>
+        <v>376</v>
       </c>
       <c r="O8" t="s">
-        <v>227</v>
+        <v>271</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>324</v>
+        <v>377</v>
       </c>
       <c r="D9" t="s">
-        <v>325</v>
+        <v>378</v>
       </c>
       <c r="M9" t="s">
-        <v>326</v>
+        <v>379</v>
       </c>
       <c r="N9" t="s">
-        <v>326</v>
+        <v>379</v>
       </c>
       <c r="O9" t="s">
-        <v>264</v>
+        <v>308</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>327</v>
+        <v>380</v>
       </c>
       <c r="D10" t="s">
-        <v>328</v>
+        <v>381</v>
       </c>
       <c r="M10" t="s">
-        <v>329</v>
+        <v>382</v>
       </c>
       <c r="N10" t="s">
-        <v>330</v>
+        <v>383</v>
+      </c>
+      <c r="O10" t="s">
+        <v>310</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>318</v>
+        <v>371</v>
       </c>
       <c r="D11" t="s">
-        <v>331</v>
+        <v>384</v>
       </c>
       <c r="M11" t="s">
-        <v>332</v>
+        <v>385</v>
       </c>
       <c r="N11" t="s">
-        <v>333</v>
+        <v>386</v>
+      </c>
+      <c r="O11" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="D12" t="s">
-        <v>318</v>
+        <v>371</v>
       </c>
       <c r="M12" t="s">
-        <v>334</v>
+        <v>387</v>
       </c>
       <c r="N12" t="s">
-        <v>335</v>
+        <v>388</v>
+      </c>
+      <c r="O12" t="s">
+        <v>314</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M13" t="s">
-        <v>336</v>
+        <v>389</v>
       </c>
       <c r="N13" t="s">
-        <v>337</v>
+        <v>390</v>
+      </c>
+      <c r="O13" t="s">
+        <v>316</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M14" t="s">
-        <v>338</v>
+        <v>391</v>
       </c>
       <c r="N14" t="s">
-        <v>339</v>
+        <v>392</v>
+      </c>
+      <c r="O14" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M15" t="s">
-        <v>340</v>
+        <v>393</v>
       </c>
       <c r="N15" t="s">
-        <v>341</v>
+        <v>394</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M16" t="s">
-        <v>342</v>
+        <v>395</v>
       </c>
       <c r="N16" t="s">
-        <v>343</v>
+        <v>396</v>
       </c>
     </row>
   </sheetData>

</xml_diff>